<commit_message>
Normalize Rev A reference designators
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -51,7 +51,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:L302"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
@@ -874,7 +874,7 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U6</t>
+          <t>02_Power_Conversion/U206</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="0">
@@ -936,7 +936,7 @@
     <row r="15">
       <c r="A15" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/U4</t>
+          <t>07_UI_Peripherals/U704</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="0">
@@ -998,7 +998,7 @@
     <row r="16">
       <c r="A16" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/U6</t>
+          <t>07_UI_Peripherals/U706</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="0">
@@ -1060,7 +1060,7 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/U1</t>
+          <t>03_ESP32_Core/U301</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="0">
@@ -1122,7 +1122,7 @@
     <row r="18">
       <c r="A18" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U10</t>
+          <t>02_Power_Conversion/U210</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="0">
@@ -1184,7 +1184,7 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U11</t>
+          <t>02_Power_Conversion/U211</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="0">
@@ -1246,7 +1246,7 @@
     <row r="20">
       <c r="A20" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/U2</t>
+          <t>07_UI_Peripherals/U702</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="0">
@@ -1308,7 +1308,7 @@
     <row r="21">
       <c r="A21" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/U2</t>
+          <t>08_Expansion/U802</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="0">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U4</t>
+          <t>02_Power_Conversion/U204</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="0">
@@ -1432,7 +1432,7 @@
     <row r="23">
       <c r="A23" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U5</t>
+          <t>02_Power_Conversion/U205</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="0">
@@ -1494,7 +1494,7 @@
     <row r="24">
       <c r="A24" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/U2</t>
+          <t>03_ESP32_Core/U302</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="0">
@@ -1556,7 +1556,7 @@
     <row r="25">
       <c r="A25" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/U1</t>
+          <t>05_Motor_Interfaces/U501</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="0">
@@ -1618,7 +1618,7 @@
     <row r="26">
       <c r="A26" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/U2</t>
+          <t>05_Motor_Interfaces/U502</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="0">
@@ -1680,7 +1680,7 @@
     <row r="27">
       <c r="A27" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/U3</t>
+          <t>05_Motor_Interfaces/U503</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="0">
@@ -1742,7 +1742,7 @@
     <row r="28">
       <c r="A28" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/U4</t>
+          <t>05_Motor_Interfaces/U504</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="0">
@@ -1804,7 +1804,7 @@
     <row r="29">
       <c r="A29" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/U5</t>
+          <t>05_Motor_Interfaces/U505</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="0">
@@ -1866,7 +1866,7 @@
     <row r="30">
       <c r="A30" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/U2</t>
+          <t>06_Relay_MasterInhibit/U602</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="0">
@@ -1928,7 +1928,7 @@
     <row r="31">
       <c r="A31" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/U3</t>
+          <t>06_Relay_MasterInhibit/U603</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="0">
@@ -1990,7 +1990,7 @@
     <row r="32">
       <c r="A32" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/U1</t>
+          <t>07_UI_Peripherals/U701</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="0">
@@ -2052,7 +2052,7 @@
     <row r="33">
       <c r="A33" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/U3</t>
+          <t>07_UI_Peripherals/U703</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="0">
@@ -2114,7 +2114,7 @@
     <row r="34">
       <c r="A34" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/Q1</t>
+          <t>01_Power_Entry/Q101</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="0">
@@ -2176,7 +2176,7 @@
     <row r="35">
       <c r="A35" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/Q2</t>
+          <t>01_Power_Entry/Q102</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="0">
@@ -2238,7 +2238,7 @@
     <row r="36">
       <c r="A36" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/Q1</t>
+          <t>06_Relay_MasterInhibit/Q601</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="0">
@@ -2300,7 +2300,7 @@
     <row r="37">
       <c r="A37" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/Q1</t>
+          <t>07_UI_Peripherals/Q701</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="0">
@@ -2362,7 +2362,7 @@
     <row r="38">
       <c r="A38" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C1</t>
+          <t>01_Power_Entry/C101</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="0">
@@ -2424,7 +2424,7 @@
     <row r="39">
       <c r="A39" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C2</t>
+          <t>01_Power_Entry/C102</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="0">
@@ -2486,7 +2486,7 @@
     <row r="40">
       <c r="A40" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C3</t>
+          <t>01_Power_Entry/C103</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="0">
@@ -2548,7 +2548,7 @@
     <row r="41">
       <c r="A41" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C4</t>
+          <t>01_Power_Entry/C104</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="0">
@@ -2610,7 +2610,7 @@
     <row r="42">
       <c r="A42" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C5</t>
+          <t>01_Power_Entry/C105</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="0">
@@ -2672,7 +2672,7 @@
     <row r="43">
       <c r="A43" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C6</t>
+          <t>01_Power_Entry/C106</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="0">
@@ -2734,7 +2734,7 @@
     <row r="44">
       <c r="A44" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C7</t>
+          <t>01_Power_Entry/C107</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="0">
@@ -2796,7 +2796,7 @@
     <row r="45">
       <c r="A45" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C8</t>
+          <t>01_Power_Entry/C108</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="0">
@@ -2858,7 +2858,7 @@
     <row r="46">
       <c r="A46" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/C9</t>
+          <t>01_Power_Entry/C109</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="0">
@@ -2920,7 +2920,7 @@
     <row r="47">
       <c r="A47" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/L1</t>
+          <t>01_Power_Entry/L101</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="0">
@@ -2982,7 +2982,7 @@
     <row r="48">
       <c r="A48" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R1</t>
+          <t>01_Power_Entry/R101</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="0">
@@ -3044,7 +3044,7 @@
     <row r="49">
       <c r="A49" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R10</t>
+          <t>01_Power_Entry/R102</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="0">
@@ -3106,7 +3106,7 @@
     <row r="50">
       <c r="A50" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R11</t>
+          <t>01_Power_Entry/R103</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="0">
@@ -3168,7 +3168,7 @@
     <row r="51">
       <c r="A51" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R12</t>
+          <t>01_Power_Entry/R104</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="0">
@@ -3230,7 +3230,7 @@
     <row r="52">
       <c r="A52" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R13</t>
+          <t>01_Power_Entry/R105</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="0">
@@ -3292,7 +3292,7 @@
     <row r="53">
       <c r="A53" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R14</t>
+          <t>01_Power_Entry/R106</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="0">
@@ -3354,7 +3354,7 @@
     <row r="54">
       <c r="A54" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R15</t>
+          <t>01_Power_Entry/R107</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="0">
@@ -3416,7 +3416,7 @@
     <row r="55">
       <c r="A55" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R16</t>
+          <t>01_Power_Entry/R108</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="0">
@@ -3478,7 +3478,7 @@
     <row r="56">
       <c r="A56" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R2</t>
+          <t>01_Power_Entry/R109</t>
         </is>
       </c>
       <c r="B56" t="inlineStr" s="0">
@@ -3540,7 +3540,7 @@
     <row r="57">
       <c r="A57" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R3</t>
+          <t>01_Power_Entry/R110</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="0">
@@ -3602,7 +3602,7 @@
     <row r="58">
       <c r="A58" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R4</t>
+          <t>01_Power_Entry/R111</t>
         </is>
       </c>
       <c r="B58" t="inlineStr" s="0">
@@ -3664,7 +3664,7 @@
     <row r="59">
       <c r="A59" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R5</t>
+          <t>01_Power_Entry/R112</t>
         </is>
       </c>
       <c r="B59" t="inlineStr" s="0">
@@ -3726,7 +3726,7 @@
     <row r="60">
       <c r="A60" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R6</t>
+          <t>01_Power_Entry/R113</t>
         </is>
       </c>
       <c r="B60" t="inlineStr" s="0">
@@ -3788,7 +3788,7 @@
     <row r="61">
       <c r="A61" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R7</t>
+          <t>01_Power_Entry/R114</t>
         </is>
       </c>
       <c r="B61" t="inlineStr" s="0">
@@ -3850,7 +3850,7 @@
     <row r="62">
       <c r="A62" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R8</t>
+          <t>01_Power_Entry/R115</t>
         </is>
       </c>
       <c r="B62" t="inlineStr" s="0">
@@ -3912,7 +3912,7 @@
     <row r="63">
       <c r="A63" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/R9</t>
+          <t>01_Power_Entry/R116</t>
         </is>
       </c>
       <c r="B63" t="inlineStr" s="0">
@@ -3974,7 +3974,7 @@
     <row r="64">
       <c r="A64" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C1</t>
+          <t>02_Power_Conversion/C201</t>
         </is>
       </c>
       <c r="B64" t="inlineStr" s="0">
@@ -4036,7 +4036,7 @@
     <row r="65">
       <c r="A65" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C10</t>
+          <t>02_Power_Conversion/C202</t>
         </is>
       </c>
       <c r="B65" t="inlineStr" s="0">
@@ -4098,7 +4098,7 @@
     <row r="66">
       <c r="A66" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C11</t>
+          <t>02_Power_Conversion/C203</t>
         </is>
       </c>
       <c r="B66" t="inlineStr" s="0">
@@ -4160,7 +4160,7 @@
     <row r="67">
       <c r="A67" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C12</t>
+          <t>02_Power_Conversion/C204</t>
         </is>
       </c>
       <c r="B67" t="inlineStr" s="0">
@@ -4222,7 +4222,7 @@
     <row r="68">
       <c r="A68" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C13</t>
+          <t>02_Power_Conversion/C205</t>
         </is>
       </c>
       <c r="B68" t="inlineStr" s="0">
@@ -4284,7 +4284,7 @@
     <row r="69">
       <c r="A69" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C14</t>
+          <t>02_Power_Conversion/C206</t>
         </is>
       </c>
       <c r="B69" t="inlineStr" s="0">
@@ -4346,7 +4346,7 @@
     <row r="70">
       <c r="A70" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C15</t>
+          <t>02_Power_Conversion/C207</t>
         </is>
       </c>
       <c r="B70" t="inlineStr" s="0">
@@ -4408,7 +4408,7 @@
     <row r="71">
       <c r="A71" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C16</t>
+          <t>02_Power_Conversion/C208</t>
         </is>
       </c>
       <c r="B71" t="inlineStr" s="0">
@@ -4470,7 +4470,7 @@
     <row r="72">
       <c r="A72" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C17</t>
+          <t>02_Power_Conversion/C209</t>
         </is>
       </c>
       <c r="B72" t="inlineStr" s="0">
@@ -4532,7 +4532,7 @@
     <row r="73">
       <c r="A73" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C18</t>
+          <t>02_Power_Conversion/C210</t>
         </is>
       </c>
       <c r="B73" t="inlineStr" s="0">
@@ -4594,7 +4594,7 @@
     <row r="74">
       <c r="A74" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C19</t>
+          <t>02_Power_Conversion/C211</t>
         </is>
       </c>
       <c r="B74" t="inlineStr" s="0">
@@ -4656,7 +4656,7 @@
     <row r="75">
       <c r="A75" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C2</t>
+          <t>02_Power_Conversion/C212</t>
         </is>
       </c>
       <c r="B75" t="inlineStr" s="0">
@@ -4718,7 +4718,7 @@
     <row r="76">
       <c r="A76" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C20</t>
+          <t>02_Power_Conversion/C213</t>
         </is>
       </c>
       <c r="B76" t="inlineStr" s="0">
@@ -4780,7 +4780,7 @@
     <row r="77">
       <c r="A77" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C21</t>
+          <t>02_Power_Conversion/C214</t>
         </is>
       </c>
       <c r="B77" t="inlineStr" s="0">
@@ -4842,7 +4842,7 @@
     <row r="78">
       <c r="A78" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C3</t>
+          <t>02_Power_Conversion/C215</t>
         </is>
       </c>
       <c r="B78" t="inlineStr" s="0">
@@ -4904,7 +4904,7 @@
     <row r="79">
       <c r="A79" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C4</t>
+          <t>02_Power_Conversion/C216</t>
         </is>
       </c>
       <c r="B79" t="inlineStr" s="0">
@@ -4966,7 +4966,7 @@
     <row r="80">
       <c r="A80" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C5</t>
+          <t>02_Power_Conversion/C217</t>
         </is>
       </c>
       <c r="B80" t="inlineStr" s="0">
@@ -5028,7 +5028,7 @@
     <row r="81">
       <c r="A81" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C6</t>
+          <t>02_Power_Conversion/C218</t>
         </is>
       </c>
       <c r="B81" t="inlineStr" s="0">
@@ -5090,7 +5090,7 @@
     <row r="82">
       <c r="A82" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C7</t>
+          <t>02_Power_Conversion/C219</t>
         </is>
       </c>
       <c r="B82" t="inlineStr" s="0">
@@ -5152,7 +5152,7 @@
     <row r="83">
       <c r="A83" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C8</t>
+          <t>02_Power_Conversion/C220</t>
         </is>
       </c>
       <c r="B83" t="inlineStr" s="0">
@@ -5214,7 +5214,7 @@
     <row r="84">
       <c r="A84" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/C9</t>
+          <t>02_Power_Conversion/C221</t>
         </is>
       </c>
       <c r="B84" t="inlineStr" s="0">
@@ -5276,7 +5276,7 @@
     <row r="85">
       <c r="A85" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/L1</t>
+          <t>02_Power_Conversion/L201</t>
         </is>
       </c>
       <c r="B85" t="inlineStr" s="0">
@@ -5338,7 +5338,7 @@
     <row r="86">
       <c r="A86" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/L2</t>
+          <t>02_Power_Conversion/L202</t>
         </is>
       </c>
       <c r="B86" t="inlineStr" s="0">
@@ -5400,7 +5400,7 @@
     <row r="87">
       <c r="A87" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R1</t>
+          <t>02_Power_Conversion/R201</t>
         </is>
       </c>
       <c r="B87" t="inlineStr" s="0">
@@ -5462,7 +5462,7 @@
     <row r="88">
       <c r="A88" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R10</t>
+          <t>02_Power_Conversion/R202</t>
         </is>
       </c>
       <c r="B88" t="inlineStr" s="0">
@@ -5524,7 +5524,7 @@
     <row r="89">
       <c r="A89" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R11</t>
+          <t>02_Power_Conversion/R203</t>
         </is>
       </c>
       <c r="B89" t="inlineStr" s="0">
@@ -5586,7 +5586,7 @@
     <row r="90">
       <c r="A90" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R12</t>
+          <t>02_Power_Conversion/R204</t>
         </is>
       </c>
       <c r="B90" t="inlineStr" s="0">
@@ -5648,7 +5648,7 @@
     <row r="91">
       <c r="A91" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R13</t>
+          <t>02_Power_Conversion/R205</t>
         </is>
       </c>
       <c r="B91" t="inlineStr" s="0">
@@ -5710,7 +5710,7 @@
     <row r="92">
       <c r="A92" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R14</t>
+          <t>02_Power_Conversion/R206</t>
         </is>
       </c>
       <c r="B92" t="inlineStr" s="0">
@@ -5772,7 +5772,7 @@
     <row r="93">
       <c r="A93" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R15</t>
+          <t>02_Power_Conversion/R207</t>
         </is>
       </c>
       <c r="B93" t="inlineStr" s="0">
@@ -5834,7 +5834,7 @@
     <row r="94">
       <c r="A94" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R16</t>
+          <t>02_Power_Conversion/R208</t>
         </is>
       </c>
       <c r="B94" t="inlineStr" s="0">
@@ -5896,7 +5896,7 @@
     <row r="95">
       <c r="A95" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R17</t>
+          <t>02_Power_Conversion/R209</t>
         </is>
       </c>
       <c r="B95" t="inlineStr" s="0">
@@ -5958,7 +5958,7 @@
     <row r="96">
       <c r="A96" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R18</t>
+          <t>02_Power_Conversion/R210</t>
         </is>
       </c>
       <c r="B96" t="inlineStr" s="0">
@@ -6020,7 +6020,7 @@
     <row r="97">
       <c r="A97" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R19</t>
+          <t>02_Power_Conversion/R211</t>
         </is>
       </c>
       <c r="B97" t="inlineStr" s="0">
@@ -6082,7 +6082,7 @@
     <row r="98">
       <c r="A98" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R2</t>
+          <t>02_Power_Conversion/R212</t>
         </is>
       </c>
       <c r="B98" t="inlineStr" s="0">
@@ -6144,7 +6144,7 @@
     <row r="99">
       <c r="A99" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R20</t>
+          <t>02_Power_Conversion/R213</t>
         </is>
       </c>
       <c r="B99" t="inlineStr" s="0">
@@ -6206,7 +6206,7 @@
     <row r="100">
       <c r="A100" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R21</t>
+          <t>02_Power_Conversion/R214</t>
         </is>
       </c>
       <c r="B100" t="inlineStr" s="0">
@@ -6268,7 +6268,7 @@
     <row r="101">
       <c r="A101" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R22</t>
+          <t>02_Power_Conversion/R215</t>
         </is>
       </c>
       <c r="B101" t="inlineStr" s="0">
@@ -6330,7 +6330,7 @@
     <row r="102">
       <c r="A102" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R23</t>
+          <t>02_Power_Conversion/R216</t>
         </is>
       </c>
       <c r="B102" t="inlineStr" s="0">
@@ -6392,7 +6392,7 @@
     <row r="103">
       <c r="A103" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R24</t>
+          <t>02_Power_Conversion/R217</t>
         </is>
       </c>
       <c r="B103" t="inlineStr" s="0">
@@ -6454,7 +6454,7 @@
     <row r="104">
       <c r="A104" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R25</t>
+          <t>02_Power_Conversion/R218</t>
         </is>
       </c>
       <c r="B104" t="inlineStr" s="0">
@@ -6516,7 +6516,7 @@
     <row r="105">
       <c r="A105" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R26</t>
+          <t>02_Power_Conversion/R219</t>
         </is>
       </c>
       <c r="B105" t="inlineStr" s="0">
@@ -6578,7 +6578,7 @@
     <row r="106">
       <c r="A106" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R27</t>
+          <t>02_Power_Conversion/R220</t>
         </is>
       </c>
       <c r="B106" t="inlineStr" s="0">
@@ -6640,7 +6640,7 @@
     <row r="107">
       <c r="A107" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R28</t>
+          <t>02_Power_Conversion/R221</t>
         </is>
       </c>
       <c r="B107" t="inlineStr" s="0">
@@ -6702,7 +6702,7 @@
     <row r="108">
       <c r="A108" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R29</t>
+          <t>02_Power_Conversion/R222</t>
         </is>
       </c>
       <c r="B108" t="inlineStr" s="0">
@@ -6764,7 +6764,7 @@
     <row r="109">
       <c r="A109" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R3</t>
+          <t>02_Power_Conversion/R223</t>
         </is>
       </c>
       <c r="B109" t="inlineStr" s="0">
@@ -6826,7 +6826,7 @@
     <row r="110">
       <c r="A110" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R30</t>
+          <t>02_Power_Conversion/R224</t>
         </is>
       </c>
       <c r="B110" t="inlineStr" s="0">
@@ -6888,7 +6888,7 @@
     <row r="111">
       <c r="A111" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R31</t>
+          <t>02_Power_Conversion/R225</t>
         </is>
       </c>
       <c r="B111" t="inlineStr" s="0">
@@ -6950,7 +6950,7 @@
     <row r="112">
       <c r="A112" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R4</t>
+          <t>02_Power_Conversion/R226</t>
         </is>
       </c>
       <c r="B112" t="inlineStr" s="0">
@@ -7012,7 +7012,7 @@
     <row r="113">
       <c r="A113" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R5</t>
+          <t>02_Power_Conversion/R227</t>
         </is>
       </c>
       <c r="B113" t="inlineStr" s="0">
@@ -7074,7 +7074,7 @@
     <row r="114">
       <c r="A114" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R6</t>
+          <t>02_Power_Conversion/R228</t>
         </is>
       </c>
       <c r="B114" t="inlineStr" s="0">
@@ -7136,7 +7136,7 @@
     <row r="115">
       <c r="A115" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R7</t>
+          <t>02_Power_Conversion/R229</t>
         </is>
       </c>
       <c r="B115" t="inlineStr" s="0">
@@ -7198,7 +7198,7 @@
     <row r="116">
       <c r="A116" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R8</t>
+          <t>02_Power_Conversion/R230</t>
         </is>
       </c>
       <c r="B116" t="inlineStr" s="0">
@@ -7260,7 +7260,7 @@
     <row r="117">
       <c r="A117" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/R9</t>
+          <t>02_Power_Conversion/R231</t>
         </is>
       </c>
       <c r="B117" t="inlineStr" s="0">
@@ -7322,7 +7322,7 @@
     <row r="118">
       <c r="A118" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/C1</t>
+          <t>03_ESP32_Core/C301</t>
         </is>
       </c>
       <c r="B118" t="inlineStr" s="0">
@@ -7384,7 +7384,7 @@
     <row r="119">
       <c r="A119" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/C2</t>
+          <t>03_ESP32_Core/C302</t>
         </is>
       </c>
       <c r="B119" t="inlineStr" s="0">
@@ -7446,7 +7446,7 @@
     <row r="120">
       <c r="A120" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/C3</t>
+          <t>03_ESP32_Core/C303</t>
         </is>
       </c>
       <c r="B120" t="inlineStr" s="0">
@@ -7508,7 +7508,7 @@
     <row r="121">
       <c r="A121" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/C4</t>
+          <t>03_ESP32_Core/C304</t>
         </is>
       </c>
       <c r="B121" t="inlineStr" s="0">
@@ -7570,7 +7570,7 @@
     <row r="122">
       <c r="A122" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/C5</t>
+          <t>03_ESP32_Core/C305</t>
         </is>
       </c>
       <c r="B122" t="inlineStr" s="0">
@@ -7632,7 +7632,7 @@
     <row r="123">
       <c r="A123" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/C6</t>
+          <t>03_ESP32_Core/C306</t>
         </is>
       </c>
       <c r="B123" t="inlineStr" s="0">
@@ -7694,7 +7694,7 @@
     <row r="124">
       <c r="A124" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/R1</t>
+          <t>03_ESP32_Core/R301</t>
         </is>
       </c>
       <c r="B124" t="inlineStr" s="0">
@@ -7756,7 +7756,7 @@
     <row r="125">
       <c r="A125" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/R2</t>
+          <t>03_ESP32_Core/R302</t>
         </is>
       </c>
       <c r="B125" t="inlineStr" s="0">
@@ -7818,7 +7818,7 @@
     <row r="126">
       <c r="A126" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/R3</t>
+          <t>03_ESP32_Core/R303</t>
         </is>
       </c>
       <c r="B126" t="inlineStr" s="0">
@@ -7880,7 +7880,7 @@
     <row r="127">
       <c r="A127" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/R4</t>
+          <t>03_ESP32_Core/R304</t>
         </is>
       </c>
       <c r="B127" t="inlineStr" s="0">
@@ -7942,7 +7942,7 @@
     <row r="128">
       <c r="A128" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/R5</t>
+          <t>03_ESP32_Core/R305</t>
         </is>
       </c>
       <c r="B128" t="inlineStr" s="0">
@@ -8004,7 +8004,7 @@
     <row r="129">
       <c r="A129" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C1</t>
+          <t>04_Safety_Inputs/C401</t>
         </is>
       </c>
       <c r="B129" t="inlineStr" s="0">
@@ -8066,7 +8066,7 @@
     <row r="130">
       <c r="A130" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C10</t>
+          <t>04_Safety_Inputs/C402</t>
         </is>
       </c>
       <c r="B130" t="inlineStr" s="0">
@@ -8128,7 +8128,7 @@
     <row r="131">
       <c r="A131" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C11</t>
+          <t>04_Safety_Inputs/C403</t>
         </is>
       </c>
       <c r="B131" t="inlineStr" s="0">
@@ -8190,7 +8190,7 @@
     <row r="132">
       <c r="A132" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C12</t>
+          <t>04_Safety_Inputs/C404</t>
         </is>
       </c>
       <c r="B132" t="inlineStr" s="0">
@@ -8252,7 +8252,7 @@
     <row r="133">
       <c r="A133" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C13</t>
+          <t>04_Safety_Inputs/C405</t>
         </is>
       </c>
       <c r="B133" t="inlineStr" s="0">
@@ -8314,7 +8314,7 @@
     <row r="134">
       <c r="A134" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C2</t>
+          <t>04_Safety_Inputs/C406</t>
         </is>
       </c>
       <c r="B134" t="inlineStr" s="0">
@@ -8376,7 +8376,7 @@
     <row r="135">
       <c r="A135" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C3</t>
+          <t>04_Safety_Inputs/C407</t>
         </is>
       </c>
       <c r="B135" t="inlineStr" s="0">
@@ -8438,7 +8438,7 @@
     <row r="136">
       <c r="A136" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C4</t>
+          <t>04_Safety_Inputs/C408</t>
         </is>
       </c>
       <c r="B136" t="inlineStr" s="0">
@@ -8500,7 +8500,7 @@
     <row r="137">
       <c r="A137" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C5</t>
+          <t>04_Safety_Inputs/C409</t>
         </is>
       </c>
       <c r="B137" t="inlineStr" s="0">
@@ -8562,7 +8562,7 @@
     <row r="138">
       <c r="A138" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C6</t>
+          <t>04_Safety_Inputs/C410</t>
         </is>
       </c>
       <c r="B138" t="inlineStr" s="0">
@@ -8624,7 +8624,7 @@
     <row r="139">
       <c r="A139" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C7</t>
+          <t>04_Safety_Inputs/C411</t>
         </is>
       </c>
       <c r="B139" t="inlineStr" s="0">
@@ -8686,7 +8686,7 @@
     <row r="140">
       <c r="A140" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C8</t>
+          <t>04_Safety_Inputs/C412</t>
         </is>
       </c>
       <c r="B140" t="inlineStr" s="0">
@@ -8748,7 +8748,7 @@
     <row r="141">
       <c r="A141" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/C9</t>
+          <t>04_Safety_Inputs/C413</t>
         </is>
       </c>
       <c r="B141" t="inlineStr" s="0">
@@ -8810,7 +8810,7 @@
     <row r="142">
       <c r="A142" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R1</t>
+          <t>04_Safety_Inputs/R401</t>
         </is>
       </c>
       <c r="B142" t="inlineStr" s="0">
@@ -8872,7 +8872,7 @@
     <row r="143">
       <c r="A143" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R10</t>
+          <t>04_Safety_Inputs/R402</t>
         </is>
       </c>
       <c r="B143" t="inlineStr" s="0">
@@ -8934,7 +8934,7 @@
     <row r="144">
       <c r="A144" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R11</t>
+          <t>04_Safety_Inputs/R403</t>
         </is>
       </c>
       <c r="B144" t="inlineStr" s="0">
@@ -8996,7 +8996,7 @@
     <row r="145">
       <c r="A145" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R12</t>
+          <t>04_Safety_Inputs/R404</t>
         </is>
       </c>
       <c r="B145" t="inlineStr" s="0">
@@ -9058,7 +9058,7 @@
     <row r="146">
       <c r="A146" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R13</t>
+          <t>04_Safety_Inputs/R405</t>
         </is>
       </c>
       <c r="B146" t="inlineStr" s="0">
@@ -9120,7 +9120,7 @@
     <row r="147">
       <c r="A147" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R14</t>
+          <t>04_Safety_Inputs/R406</t>
         </is>
       </c>
       <c r="B147" t="inlineStr" s="0">
@@ -9182,7 +9182,7 @@
     <row r="148">
       <c r="A148" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R15</t>
+          <t>04_Safety_Inputs/R407</t>
         </is>
       </c>
       <c r="B148" t="inlineStr" s="0">
@@ -9244,7 +9244,7 @@
     <row r="149">
       <c r="A149" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R16</t>
+          <t>04_Safety_Inputs/R408</t>
         </is>
       </c>
       <c r="B149" t="inlineStr" s="0">
@@ -9306,7 +9306,7 @@
     <row r="150">
       <c r="A150" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R17</t>
+          <t>04_Safety_Inputs/R409</t>
         </is>
       </c>
       <c r="B150" t="inlineStr" s="0">
@@ -9368,7 +9368,7 @@
     <row r="151">
       <c r="A151" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R18</t>
+          <t>04_Safety_Inputs/R410</t>
         </is>
       </c>
       <c r="B151" t="inlineStr" s="0">
@@ -9430,7 +9430,7 @@
     <row r="152">
       <c r="A152" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R19</t>
+          <t>04_Safety_Inputs/R411</t>
         </is>
       </c>
       <c r="B152" t="inlineStr" s="0">
@@ -9492,7 +9492,7 @@
     <row r="153">
       <c r="A153" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R2</t>
+          <t>04_Safety_Inputs/R412</t>
         </is>
       </c>
       <c r="B153" t="inlineStr" s="0">
@@ -9554,7 +9554,7 @@
     <row r="154">
       <c r="A154" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R20</t>
+          <t>04_Safety_Inputs/R413</t>
         </is>
       </c>
       <c r="B154" t="inlineStr" s="0">
@@ -9616,7 +9616,7 @@
     <row r="155">
       <c r="A155" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R21</t>
+          <t>04_Safety_Inputs/R414</t>
         </is>
       </c>
       <c r="B155" t="inlineStr" s="0">
@@ -9678,7 +9678,7 @@
     <row r="156">
       <c r="A156" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R22</t>
+          <t>04_Safety_Inputs/R415</t>
         </is>
       </c>
       <c r="B156" t="inlineStr" s="0">
@@ -9740,7 +9740,7 @@
     <row r="157">
       <c r="A157" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R23</t>
+          <t>04_Safety_Inputs/R416</t>
         </is>
       </c>
       <c r="B157" t="inlineStr" s="0">
@@ -9802,7 +9802,7 @@
     <row r="158">
       <c r="A158" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R24</t>
+          <t>04_Safety_Inputs/R417</t>
         </is>
       </c>
       <c r="B158" t="inlineStr" s="0">
@@ -9864,7 +9864,7 @@
     <row r="159">
       <c r="A159" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R3</t>
+          <t>04_Safety_Inputs/R418</t>
         </is>
       </c>
       <c r="B159" t="inlineStr" s="0">
@@ -9926,7 +9926,7 @@
     <row r="160">
       <c r="A160" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R4</t>
+          <t>04_Safety_Inputs/R419</t>
         </is>
       </c>
       <c r="B160" t="inlineStr" s="0">
@@ -9988,7 +9988,7 @@
     <row r="161">
       <c r="A161" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R5</t>
+          <t>04_Safety_Inputs/R420</t>
         </is>
       </c>
       <c r="B161" t="inlineStr" s="0">
@@ -10050,7 +10050,7 @@
     <row r="162">
       <c r="A162" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R6</t>
+          <t>04_Safety_Inputs/R421</t>
         </is>
       </c>
       <c r="B162" t="inlineStr" s="0">
@@ -10112,7 +10112,7 @@
     <row r="163">
       <c r="A163" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R7</t>
+          <t>04_Safety_Inputs/R422</t>
         </is>
       </c>
       <c r="B163" t="inlineStr" s="0">
@@ -10174,7 +10174,7 @@
     <row r="164">
       <c r="A164" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R8</t>
+          <t>04_Safety_Inputs/R423</t>
         </is>
       </c>
       <c r="B164" t="inlineStr" s="0">
@@ -10236,7 +10236,7 @@
     <row r="165">
       <c r="A165" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/R9</t>
+          <t>04_Safety_Inputs/R424</t>
         </is>
       </c>
       <c r="B165" t="inlineStr" s="0">
@@ -10298,7 +10298,7 @@
     <row r="166">
       <c r="A166" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/C1</t>
+          <t>05_Motor_Interfaces/C501</t>
         </is>
       </c>
       <c r="B166" t="inlineStr" s="0">
@@ -10360,7 +10360,7 @@
     <row r="167">
       <c r="A167" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/C2</t>
+          <t>05_Motor_Interfaces/C502</t>
         </is>
       </c>
       <c r="B167" t="inlineStr" s="0">
@@ -10422,7 +10422,7 @@
     <row r="168">
       <c r="A168" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/C3</t>
+          <t>05_Motor_Interfaces/C503</t>
         </is>
       </c>
       <c r="B168" t="inlineStr" s="0">
@@ -10484,7 +10484,7 @@
     <row r="169">
       <c r="A169" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/C4</t>
+          <t>05_Motor_Interfaces/C504</t>
         </is>
       </c>
       <c r="B169" t="inlineStr" s="0">
@@ -10546,7 +10546,7 @@
     <row r="170">
       <c r="A170" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/C5</t>
+          <t>05_Motor_Interfaces/C505</t>
         </is>
       </c>
       <c r="B170" t="inlineStr" s="0">
@@ -10608,7 +10608,7 @@
     <row r="171">
       <c r="A171" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/C6</t>
+          <t>05_Motor_Interfaces/C506</t>
         </is>
       </c>
       <c r="B171" t="inlineStr" s="0">
@@ -10670,7 +10670,7 @@
     <row r="172">
       <c r="A172" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R1</t>
+          <t>05_Motor_Interfaces/R501</t>
         </is>
       </c>
       <c r="B172" t="inlineStr" s="0">
@@ -10732,7 +10732,7 @@
     <row r="173">
       <c r="A173" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R10</t>
+          <t>05_Motor_Interfaces/R502</t>
         </is>
       </c>
       <c r="B173" t="inlineStr" s="0">
@@ -10794,7 +10794,7 @@
     <row r="174">
       <c r="A174" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R11</t>
+          <t>05_Motor_Interfaces/R503</t>
         </is>
       </c>
       <c r="B174" t="inlineStr" s="0">
@@ -10856,7 +10856,7 @@
     <row r="175">
       <c r="A175" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R12</t>
+          <t>05_Motor_Interfaces/R504</t>
         </is>
       </c>
       <c r="B175" t="inlineStr" s="0">
@@ -10918,7 +10918,7 @@
     <row r="176">
       <c r="A176" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R13</t>
+          <t>05_Motor_Interfaces/R505</t>
         </is>
       </c>
       <c r="B176" t="inlineStr" s="0">
@@ -10980,7 +10980,7 @@
     <row r="177">
       <c r="A177" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R14</t>
+          <t>05_Motor_Interfaces/R506</t>
         </is>
       </c>
       <c r="B177" t="inlineStr" s="0">
@@ -11042,7 +11042,7 @@
     <row r="178">
       <c r="A178" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R15</t>
+          <t>05_Motor_Interfaces/R507</t>
         </is>
       </c>
       <c r="B178" t="inlineStr" s="0">
@@ -11104,7 +11104,7 @@
     <row r="179">
       <c r="A179" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R16</t>
+          <t>05_Motor_Interfaces/R508</t>
         </is>
       </c>
       <c r="B179" t="inlineStr" s="0">
@@ -11166,7 +11166,7 @@
     <row r="180">
       <c r="A180" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R17</t>
+          <t>05_Motor_Interfaces/R509</t>
         </is>
       </c>
       <c r="B180" t="inlineStr" s="0">
@@ -11228,7 +11228,7 @@
     <row r="181">
       <c r="A181" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R18</t>
+          <t>05_Motor_Interfaces/R510</t>
         </is>
       </c>
       <c r="B181" t="inlineStr" s="0">
@@ -11290,7 +11290,7 @@
     <row r="182">
       <c r="A182" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R19</t>
+          <t>05_Motor_Interfaces/R511</t>
         </is>
       </c>
       <c r="B182" t="inlineStr" s="0">
@@ -11352,7 +11352,7 @@
     <row r="183">
       <c r="A183" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R2</t>
+          <t>05_Motor_Interfaces/R512</t>
         </is>
       </c>
       <c r="B183" t="inlineStr" s="0">
@@ -11414,7 +11414,7 @@
     <row r="184">
       <c r="A184" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R20</t>
+          <t>05_Motor_Interfaces/R513</t>
         </is>
       </c>
       <c r="B184" t="inlineStr" s="0">
@@ -11476,7 +11476,7 @@
     <row r="185">
       <c r="A185" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R21</t>
+          <t>05_Motor_Interfaces/R514</t>
         </is>
       </c>
       <c r="B185" t="inlineStr" s="0">
@@ -11538,7 +11538,7 @@
     <row r="186">
       <c r="A186" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R22</t>
+          <t>05_Motor_Interfaces/R515</t>
         </is>
       </c>
       <c r="B186" t="inlineStr" s="0">
@@ -11600,7 +11600,7 @@
     <row r="187">
       <c r="A187" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R23</t>
+          <t>05_Motor_Interfaces/R516</t>
         </is>
       </c>
       <c r="B187" t="inlineStr" s="0">
@@ -11662,7 +11662,7 @@
     <row r="188">
       <c r="A188" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R24</t>
+          <t>05_Motor_Interfaces/R517</t>
         </is>
       </c>
       <c r="B188" t="inlineStr" s="0">
@@ -11724,7 +11724,7 @@
     <row r="189">
       <c r="A189" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R25</t>
+          <t>05_Motor_Interfaces/R518</t>
         </is>
       </c>
       <c r="B189" t="inlineStr" s="0">
@@ -11786,7 +11786,7 @@
     <row r="190">
       <c r="A190" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R26</t>
+          <t>05_Motor_Interfaces/R519</t>
         </is>
       </c>
       <c r="B190" t="inlineStr" s="0">
@@ -11848,7 +11848,7 @@
     <row r="191">
       <c r="A191" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R27</t>
+          <t>05_Motor_Interfaces/R520</t>
         </is>
       </c>
       <c r="B191" t="inlineStr" s="0">
@@ -11910,7 +11910,7 @@
     <row r="192">
       <c r="A192" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R28</t>
+          <t>05_Motor_Interfaces/R521</t>
         </is>
       </c>
       <c r="B192" t="inlineStr" s="0">
@@ -11972,7 +11972,7 @@
     <row r="193">
       <c r="A193" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R3</t>
+          <t>05_Motor_Interfaces/R522</t>
         </is>
       </c>
       <c r="B193" t="inlineStr" s="0">
@@ -12034,7 +12034,7 @@
     <row r="194">
       <c r="A194" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R4</t>
+          <t>05_Motor_Interfaces/R523</t>
         </is>
       </c>
       <c r="B194" t="inlineStr" s="0">
@@ -12096,7 +12096,7 @@
     <row r="195">
       <c r="A195" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R5</t>
+          <t>05_Motor_Interfaces/R524</t>
         </is>
       </c>
       <c r="B195" t="inlineStr" s="0">
@@ -12158,7 +12158,7 @@
     <row r="196">
       <c r="A196" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R6</t>
+          <t>05_Motor_Interfaces/R525</t>
         </is>
       </c>
       <c r="B196" t="inlineStr" s="0">
@@ -12220,7 +12220,7 @@
     <row r="197">
       <c r="A197" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R7</t>
+          <t>05_Motor_Interfaces/R526</t>
         </is>
       </c>
       <c r="B197" t="inlineStr" s="0">
@@ -12282,7 +12282,7 @@
     <row r="198">
       <c r="A198" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R8</t>
+          <t>05_Motor_Interfaces/R527</t>
         </is>
       </c>
       <c r="B198" t="inlineStr" s="0">
@@ -12344,7 +12344,7 @@
     <row r="199">
       <c r="A199" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/R9</t>
+          <t>05_Motor_Interfaces/R528</t>
         </is>
       </c>
       <c r="B199" t="inlineStr" s="0">
@@ -12406,7 +12406,7 @@
     <row r="200">
       <c r="A200" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/C1</t>
+          <t>06_Relay_MasterInhibit/C601</t>
         </is>
       </c>
       <c r="B200" t="inlineStr" s="0">
@@ -12468,7 +12468,7 @@
     <row r="201">
       <c r="A201" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R1</t>
+          <t>06_Relay_MasterInhibit/R601</t>
         </is>
       </c>
       <c r="B201" t="inlineStr" s="0">
@@ -12530,7 +12530,7 @@
     <row r="202">
       <c r="A202" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R10</t>
+          <t>06_Relay_MasterInhibit/R602</t>
         </is>
       </c>
       <c r="B202" t="inlineStr" s="0">
@@ -12592,7 +12592,7 @@
     <row r="203">
       <c r="A203" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R2</t>
+          <t>06_Relay_MasterInhibit/R603</t>
         </is>
       </c>
       <c r="B203" t="inlineStr" s="0">
@@ -12654,7 +12654,7 @@
     <row r="204">
       <c r="A204" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R3</t>
+          <t>06_Relay_MasterInhibit/R604</t>
         </is>
       </c>
       <c r="B204" t="inlineStr" s="0">
@@ -12716,7 +12716,7 @@
     <row r="205">
       <c r="A205" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R4</t>
+          <t>06_Relay_MasterInhibit/R605</t>
         </is>
       </c>
       <c r="B205" t="inlineStr" s="0">
@@ -12778,7 +12778,7 @@
     <row r="206">
       <c r="A206" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R5</t>
+          <t>06_Relay_MasterInhibit/R606</t>
         </is>
       </c>
       <c r="B206" t="inlineStr" s="0">
@@ -12840,7 +12840,7 @@
     <row r="207">
       <c r="A207" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R6</t>
+          <t>06_Relay_MasterInhibit/R607</t>
         </is>
       </c>
       <c r="B207" t="inlineStr" s="0">
@@ -12902,7 +12902,7 @@
     <row r="208">
       <c r="A208" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R7</t>
+          <t>06_Relay_MasterInhibit/R608</t>
         </is>
       </c>
       <c r="B208" t="inlineStr" s="0">
@@ -12964,7 +12964,7 @@
     <row r="209">
       <c r="A209" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R8</t>
+          <t>06_Relay_MasterInhibit/R609</t>
         </is>
       </c>
       <c r="B209" t="inlineStr" s="0">
@@ -13026,7 +13026,7 @@
     <row r="210">
       <c r="A210" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/R9</t>
+          <t>06_Relay_MasterInhibit/R610</t>
         </is>
       </c>
       <c r="B210" t="inlineStr" s="0">
@@ -13088,7 +13088,7 @@
     <row r="211">
       <c r="A211" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/C1</t>
+          <t>07_UI_Peripherals/C701</t>
         </is>
       </c>
       <c r="B211" t="inlineStr" s="0">
@@ -13150,7 +13150,7 @@
     <row r="212">
       <c r="A212" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/R1</t>
+          <t>07_UI_Peripherals/R701</t>
         </is>
       </c>
       <c r="B212" t="inlineStr" s="0">
@@ -13212,7 +13212,7 @@
     <row r="213">
       <c r="A213" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/R2</t>
+          <t>07_UI_Peripherals/R702</t>
         </is>
       </c>
       <c r="B213" t="inlineStr" s="0">
@@ -13274,7 +13274,7 @@
     <row r="214">
       <c r="A214" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/R3</t>
+          <t>07_UI_Peripherals/R703</t>
         </is>
       </c>
       <c r="B214" t="inlineStr" s="0">
@@ -13336,7 +13336,7 @@
     <row r="215">
       <c r="A215" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/C1</t>
+          <t>08_Expansion/C801</t>
         </is>
       </c>
       <c r="B215" t="inlineStr" s="0">
@@ -13398,7 +13398,7 @@
     <row r="216">
       <c r="A216" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/C2</t>
+          <t>08_Expansion/C802</t>
         </is>
       </c>
       <c r="B216" t="inlineStr" s="0">
@@ -13460,7 +13460,7 @@
     <row r="217">
       <c r="A217" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/C3</t>
+          <t>08_Expansion/C803</t>
         </is>
       </c>
       <c r="B217" t="inlineStr" s="0">
@@ -13522,7 +13522,7 @@
     <row r="218">
       <c r="A218" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/FB1</t>
+          <t>08_Expansion/FB801</t>
         </is>
       </c>
       <c r="B218" t="inlineStr" s="0">
@@ -13584,7 +13584,7 @@
     <row r="219">
       <c r="A219" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/R1</t>
+          <t>08_Expansion/R801</t>
         </is>
       </c>
       <c r="B219" t="inlineStr" s="0">
@@ -13646,7 +13646,7 @@
     <row r="220">
       <c r="A220" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/R2</t>
+          <t>08_Expansion/R802</t>
         </is>
       </c>
       <c r="B220" t="inlineStr" s="0">
@@ -13708,7 +13708,7 @@
     <row r="221">
       <c r="A221" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/R3</t>
+          <t>08_Expansion/R803</t>
         </is>
       </c>
       <c r="B221" t="inlineStr" s="0">
@@ -13770,7 +13770,7 @@
     <row r="222">
       <c r="A222" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/R4</t>
+          <t>08_Expansion/R804</t>
         </is>
       </c>
       <c r="B222" t="inlineStr" s="0">
@@ -13832,7 +13832,7 @@
     <row r="223">
       <c r="A223" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/R5</t>
+          <t>08_Expansion/R805</t>
         </is>
       </c>
       <c r="B223" t="inlineStr" s="0">
@@ -13894,7 +13894,7 @@
     <row r="224">
       <c r="A224" t="inlineStr" s="0">
         <is>
-          <t>09_Connectors_Test/C1</t>
+          <t>09_Connectors_Test/C901</t>
         </is>
       </c>
       <c r="B224" t="inlineStr" s="0">
@@ -13956,7 +13956,7 @@
     <row r="225">
       <c r="A225" t="inlineStr" s="0">
         <is>
-          <t>09_Connectors_Test/R1</t>
+          <t>09_Connectors_Test/R901</t>
         </is>
       </c>
       <c r="B225" t="inlineStr" s="0">
@@ -14018,7 +14018,7 @@
     <row r="226">
       <c r="A226" t="inlineStr" s="0">
         <is>
-          <t>09_Connectors_Test/R2</t>
+          <t>09_Connectors_Test/R902</t>
         </is>
       </c>
       <c r="B226" t="inlineStr" s="0">
@@ -14080,7 +14080,7 @@
     <row r="227">
       <c r="A227" t="inlineStr" s="0">
         <is>
-          <t>09_Connectors_Test/R3</t>
+          <t>09_Connectors_Test/R903</t>
         </is>
       </c>
       <c r="B227" t="inlineStr" s="0">
@@ -14142,7 +14142,7 @@
     <row r="228">
       <c r="A228" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/U1</t>
+          <t>01_Power_Entry/U101</t>
         </is>
       </c>
       <c r="B228" t="inlineStr" s="0">
@@ -14204,7 +14204,7 @@
     <row r="229">
       <c r="A229" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/U2</t>
+          <t>01_Power_Entry/U102</t>
         </is>
       </c>
       <c r="B229" t="inlineStr" s="0">
@@ -14266,7 +14266,7 @@
     <row r="230">
       <c r="A230" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U1</t>
+          <t>02_Power_Conversion/U201</t>
         </is>
       </c>
       <c r="B230" t="inlineStr" s="0">
@@ -14328,7 +14328,7 @@
     <row r="231">
       <c r="A231" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U12</t>
+          <t>02_Power_Conversion/U202</t>
         </is>
       </c>
       <c r="B231" t="inlineStr" s="0">
@@ -14390,7 +14390,7 @@
     <row r="232">
       <c r="A232" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U13</t>
+          <t>02_Power_Conversion/U203</t>
         </is>
       </c>
       <c r="B232" t="inlineStr" s="0">
@@ -14452,7 +14452,7 @@
     <row r="233">
       <c r="A233" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U2</t>
+          <t>02_Power_Conversion/U208</t>
         </is>
       </c>
       <c r="B233" t="inlineStr" s="0">
@@ -14514,7 +14514,7 @@
     <row r="234">
       <c r="A234" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U3</t>
+          <t>02_Power_Conversion/U209</t>
         </is>
       </c>
       <c r="B234" t="inlineStr" s="0">
@@ -14576,7 +14576,7 @@
     <row r="235">
       <c r="A235" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U8</t>
+          <t>02_Power_Conversion/U212</t>
         </is>
       </c>
       <c r="B235" t="inlineStr" s="0">
@@ -14638,7 +14638,7 @@
     <row r="236">
       <c r="A236" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U9</t>
+          <t>02_Power_Conversion/U213</t>
         </is>
       </c>
       <c r="B236" t="inlineStr" s="0">
@@ -14700,7 +14700,7 @@
     <row r="237">
       <c r="A237" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/U1</t>
+          <t>08_Expansion/U801</t>
         </is>
       </c>
       <c r="B237" t="inlineStr" s="0">
@@ -14762,7 +14762,7 @@
     <row r="238">
       <c r="A238" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/D1</t>
+          <t>01_Power_Entry/D101</t>
         </is>
       </c>
       <c r="B238" t="inlineStr" s="0">
@@ -14824,7 +14824,7 @@
     <row r="239">
       <c r="A239" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/D2</t>
+          <t>01_Power_Entry/D102</t>
         </is>
       </c>
       <c r="B239" t="inlineStr" s="0">
@@ -14886,7 +14886,7 @@
     <row r="240">
       <c r="A240" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/D3</t>
+          <t>01_Power_Entry/D103</t>
         </is>
       </c>
       <c r="B240" t="inlineStr" s="0">
@@ -14948,7 +14948,7 @@
     <row r="241">
       <c r="A241" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/D4</t>
+          <t>01_Power_Entry/D104</t>
         </is>
       </c>
       <c r="B241" t="inlineStr" s="0">
@@ -15010,7 +15010,7 @@
     <row r="242">
       <c r="A242" t="inlineStr" s="0">
         <is>
-          <t>01_Power_Entry/F1</t>
+          <t>01_Power_Entry/F101</t>
         </is>
       </c>
       <c r="B242" t="inlineStr" s="0">
@@ -15072,7 +15072,7 @@
     <row r="243">
       <c r="A243" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D1</t>
+          <t>02_Power_Conversion/D201</t>
         </is>
       </c>
       <c r="B243" t="inlineStr" s="0">
@@ -15134,7 +15134,7 @@
     <row r="244">
       <c r="A244" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D10</t>
+          <t>02_Power_Conversion/D202</t>
         </is>
       </c>
       <c r="B244" t="inlineStr" s="0">
@@ -15196,7 +15196,7 @@
     <row r="245">
       <c r="A245" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D2</t>
+          <t>02_Power_Conversion/D203</t>
         </is>
       </c>
       <c r="B245" t="inlineStr" s="0">
@@ -15258,7 +15258,7 @@
     <row r="246">
       <c r="A246" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D3</t>
+          <t>02_Power_Conversion/D204</t>
         </is>
       </c>
       <c r="B246" t="inlineStr" s="0">
@@ -15320,7 +15320,7 @@
     <row r="247">
       <c r="A247" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D4</t>
+          <t>02_Power_Conversion/D205</t>
         </is>
       </c>
       <c r="B247" t="inlineStr" s="0">
@@ -15382,7 +15382,7 @@
     <row r="248">
       <c r="A248" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D5</t>
+          <t>02_Power_Conversion/D206</t>
         </is>
       </c>
       <c r="B248" t="inlineStr" s="0">
@@ -15444,7 +15444,7 @@
     <row r="249">
       <c r="A249" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D6</t>
+          <t>02_Power_Conversion/D207</t>
         </is>
       </c>
       <c r="B249" t="inlineStr" s="0">
@@ -15506,7 +15506,7 @@
     <row r="250">
       <c r="A250" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D7</t>
+          <t>02_Power_Conversion/D208</t>
         </is>
       </c>
       <c r="B250" t="inlineStr" s="0">
@@ -15568,7 +15568,7 @@
     <row r="251">
       <c r="A251" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D8</t>
+          <t>02_Power_Conversion/D209</t>
         </is>
       </c>
       <c r="B251" t="inlineStr" s="0">
@@ -15630,7 +15630,7 @@
     <row r="252">
       <c r="A252" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/D9</t>
+          <t>02_Power_Conversion/D210</t>
         </is>
       </c>
       <c r="B252" t="inlineStr" s="0">
@@ -15692,7 +15692,7 @@
     <row r="253">
       <c r="A253" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/D1</t>
+          <t>04_Safety_Inputs/D401</t>
         </is>
       </c>
       <c r="B253" t="inlineStr" s="0">
@@ -15754,7 +15754,7 @@
     <row r="254">
       <c r="A254" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/D2</t>
+          <t>04_Safety_Inputs/D402</t>
         </is>
       </c>
       <c r="B254" t="inlineStr" s="0">
@@ -15816,7 +15816,7 @@
     <row r="255">
       <c r="A255" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/D3</t>
+          <t>04_Safety_Inputs/D403</t>
         </is>
       </c>
       <c r="B255" t="inlineStr" s="0">
@@ -15878,7 +15878,7 @@
     <row r="256">
       <c r="A256" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/D4</t>
+          <t>04_Safety_Inputs/D404</t>
         </is>
       </c>
       <c r="B256" t="inlineStr" s="0">
@@ -15940,7 +15940,7 @@
     <row r="257">
       <c r="A257" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/D5</t>
+          <t>04_Safety_Inputs/D405</t>
         </is>
       </c>
       <c r="B257" t="inlineStr" s="0">
@@ -16002,7 +16002,7 @@
     <row r="258">
       <c r="A258" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/D6</t>
+          <t>04_Safety_Inputs/D406</t>
         </is>
       </c>
       <c r="B258" t="inlineStr" s="0">
@@ -16064,7 +16064,7 @@
     <row r="259">
       <c r="A259" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/D7</t>
+          <t>04_Safety_Inputs/D407</t>
         </is>
       </c>
       <c r="B259" t="inlineStr" s="0">
@@ -16126,7 +16126,7 @@
     <row r="260">
       <c r="A260" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D1</t>
+          <t>05_Motor_Interfaces/D501</t>
         </is>
       </c>
       <c r="B260" t="inlineStr" s="0">
@@ -16188,7 +16188,7 @@
     <row r="261">
       <c r="A261" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D2</t>
+          <t>05_Motor_Interfaces/D502</t>
         </is>
       </c>
       <c r="B261" t="inlineStr" s="0">
@@ -16250,7 +16250,7 @@
     <row r="262">
       <c r="A262" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D3</t>
+          <t>05_Motor_Interfaces/D503</t>
         </is>
       </c>
       <c r="B262" t="inlineStr" s="0">
@@ -16312,7 +16312,7 @@
     <row r="263">
       <c r="A263" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D4</t>
+          <t>05_Motor_Interfaces/D504</t>
         </is>
       </c>
       <c r="B263" t="inlineStr" s="0">
@@ -16374,7 +16374,7 @@
     <row r="264">
       <c r="A264" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D5</t>
+          <t>05_Motor_Interfaces/D505</t>
         </is>
       </c>
       <c r="B264" t="inlineStr" s="0">
@@ -16436,7 +16436,7 @@
     <row r="265">
       <c r="A265" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D6</t>
+          <t>05_Motor_Interfaces/D506</t>
         </is>
       </c>
       <c r="B265" t="inlineStr" s="0">
@@ -16498,7 +16498,7 @@
     <row r="266">
       <c r="A266" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D7</t>
+          <t>05_Motor_Interfaces/D507</t>
         </is>
       </c>
       <c r="B266" t="inlineStr" s="0">
@@ -16560,7 +16560,7 @@
     <row r="267">
       <c r="A267" t="inlineStr" s="0">
         <is>
-          <t>05_Motor_Interfaces/D8</t>
+          <t>05_Motor_Interfaces/D508</t>
         </is>
       </c>
       <c r="B267" t="inlineStr" s="0">
@@ -16622,7 +16622,7 @@
     <row r="268">
       <c r="A268" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/D1</t>
+          <t>06_Relay_MasterInhibit/D601</t>
         </is>
       </c>
       <c r="B268" t="inlineStr" s="0">
@@ -16684,7 +16684,7 @@
     <row r="269">
       <c r="A269" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/D1</t>
+          <t>08_Expansion/D801</t>
         </is>
       </c>
       <c r="B269" t="inlineStr" s="0">
@@ -16746,7 +16746,7 @@
     <row r="270">
       <c r="A270" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/D2</t>
+          <t>08_Expansion/D802</t>
         </is>
       </c>
       <c r="B270" t="inlineStr" s="0">
@@ -16808,7 +16808,7 @@
     <row r="271">
       <c r="A271" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/D3</t>
+          <t>08_Expansion/D803</t>
         </is>
       </c>
       <c r="B271" t="inlineStr" s="0">
@@ -16870,7 +16870,7 @@
     <row r="272">
       <c r="A272" t="inlineStr" s="0">
         <is>
-          <t>09_Connectors_Test/D1</t>
+          <t>09_Connectors_Test/D901</t>
         </is>
       </c>
       <c r="B272" t="inlineStr" s="0">
@@ -16932,7 +16932,7 @@
     <row r="273">
       <c r="A273" t="inlineStr" s="0">
         <is>
-          <t>09_Connectors_Test/D2</t>
+          <t>09_Connectors_Test/D902</t>
         </is>
       </c>
       <c r="B273" t="inlineStr" s="0">
@@ -16994,7 +16994,7 @@
     <row r="274">
       <c r="A274" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/K1</t>
+          <t>06_Relay_MasterInhibit/K601</t>
         </is>
       </c>
       <c r="B274" t="inlineStr" s="0">
@@ -17056,7 +17056,7 @@
     <row r="275">
       <c r="A275" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U1AB</t>
+          <t>04_Safety_Inputs/U401AB</t>
         </is>
       </c>
       <c r="B275" t="inlineStr" s="0">
@@ -17118,7 +17118,7 @@
     <row r="276">
       <c r="A276" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U1CD</t>
+          <t>04_Safety_Inputs/U401CD</t>
         </is>
       </c>
       <c r="B276" t="inlineStr" s="0">
@@ -17180,7 +17180,7 @@
     <row r="277">
       <c r="A277" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U2AB</t>
+          <t>04_Safety_Inputs/U402AB</t>
         </is>
       </c>
       <c r="B277" t="inlineStr" s="0">
@@ -17242,7 +17242,7 @@
     <row r="278">
       <c r="A278" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U2CD</t>
+          <t>04_Safety_Inputs/U402CD</t>
         </is>
       </c>
       <c r="B278" t="inlineStr" s="0">
@@ -17304,7 +17304,7 @@
     <row r="279">
       <c r="A279" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U3AB</t>
+          <t>04_Safety_Inputs/U403AB</t>
         </is>
       </c>
       <c r="B279" t="inlineStr" s="0">
@@ -17366,7 +17366,7 @@
     <row r="280">
       <c r="A280" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U3C</t>
+          <t>04_Safety_Inputs/U403C</t>
         </is>
       </c>
       <c r="B280" t="inlineStr" s="0">
@@ -17428,7 +17428,7 @@
     <row r="281">
       <c r="A281" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U3D</t>
+          <t>04_Safety_Inputs/U403D</t>
         </is>
       </c>
       <c r="B281" t="inlineStr" s="0">
@@ -17490,7 +17490,7 @@
     <row r="282">
       <c r="A282" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U4</t>
+          <t>04_Safety_Inputs/U404</t>
         </is>
       </c>
       <c r="B282" t="inlineStr" s="0">
@@ -17552,7 +17552,7 @@
     <row r="283">
       <c r="A283" t="inlineStr" s="0">
         <is>
-          <t>04_Safety_Inputs/U5</t>
+          <t>04_Safety_Inputs/U405</t>
         </is>
       </c>
       <c r="B283" t="inlineStr" s="0">
@@ -17614,7 +17614,7 @@
     <row r="284">
       <c r="A284" t="inlineStr" s="0">
         <is>
-          <t>02_Power_Conversion/U7</t>
+          <t>02_Power_Conversion/U207</t>
         </is>
       </c>
       <c r="B284" t="inlineStr" s="0">
@@ -17676,7 +17676,7 @@
     <row r="285">
       <c r="A285" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/U5</t>
+          <t>07_UI_Peripherals/U705</t>
         </is>
       </c>
       <c r="B285" t="inlineStr" s="0">
@@ -17738,7 +17738,7 @@
     <row r="286">
       <c r="A286" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/U7</t>
+          <t>07_UI_Peripherals/U707</t>
         </is>
       </c>
       <c r="B286" t="inlineStr" s="0">
@@ -17800,7 +17800,7 @@
     <row r="287">
       <c r="A287" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/TP1</t>
+          <t>07_UI_Peripherals/TP701</t>
         </is>
       </c>
       <c r="B287" t="inlineStr" s="0">
@@ -17862,7 +17862,7 @@
     <row r="288">
       <c r="A288" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/TP2</t>
+          <t>07_UI_Peripherals/TP702</t>
         </is>
       </c>
       <c r="B288" t="inlineStr" s="0">
@@ -17924,7 +17924,7 @@
     <row r="289">
       <c r="A289" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/TP3</t>
+          <t>07_UI_Peripherals/TP703</t>
         </is>
       </c>
       <c r="B289" t="inlineStr" s="0">
@@ -17986,7 +17986,7 @@
     <row r="290">
       <c r="A290" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/TP4</t>
+          <t>07_UI_Peripherals/TP704</t>
         </is>
       </c>
       <c r="B290" t="inlineStr" s="0">
@@ -18048,7 +18048,7 @@
     <row r="291">
       <c r="A291" t="inlineStr" s="0">
         <is>
-          <t>07_UI_Peripherals/TP5</t>
+          <t>07_UI_Peripherals/TP705</t>
         </is>
       </c>
       <c r="B291" t="inlineStr" s="0">
@@ -18110,7 +18110,7 @@
     <row r="292">
       <c r="A292" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/TP1</t>
+          <t>08_Expansion/TP801</t>
         </is>
       </c>
       <c r="B292" t="inlineStr" s="0">
@@ -18172,7 +18172,7 @@
     <row r="293">
       <c r="A293" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/TP2</t>
+          <t>08_Expansion/TP802</t>
         </is>
       </c>
       <c r="B293" t="inlineStr" s="0">
@@ -18234,7 +18234,7 @@
     <row r="294">
       <c r="A294" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/TP3</t>
+          <t>08_Expansion/TP803</t>
         </is>
       </c>
       <c r="B294" t="inlineStr" s="0">
@@ -18296,7 +18296,7 @@
     <row r="295">
       <c r="A295" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/TP4</t>
+          <t>08_Expansion/TP804</t>
         </is>
       </c>
       <c r="B295" t="inlineStr" s="0">
@@ -18358,7 +18358,7 @@
     <row r="296">
       <c r="A296" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/TP5</t>
+          <t>08_Expansion/TP805</t>
         </is>
       </c>
       <c r="B296" t="inlineStr" s="0">
@@ -18420,7 +18420,7 @@
     <row r="297">
       <c r="A297" t="inlineStr" s="0">
         <is>
-          <t>08_Expansion/TP6</t>
+          <t>08_Expansion/TP806</t>
         </is>
       </c>
       <c r="B297" t="inlineStr" s="0">
@@ -18544,7 +18544,7 @@
     <row r="299">
       <c r="A299" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/U3</t>
+          <t>03_ESP32_Core/U303</t>
         </is>
       </c>
       <c r="B299" t="inlineStr" s="0">
@@ -18606,7 +18606,7 @@
     <row r="300">
       <c r="A300" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/SW1</t>
+          <t>03_ESP32_Core/SW301</t>
         </is>
       </c>
       <c r="B300" t="inlineStr" s="0">
@@ -18668,7 +18668,7 @@
     <row r="301">
       <c r="A301" t="inlineStr" s="0">
         <is>
-          <t>03_ESP32_Core/SW2</t>
+          <t>03_ESP32_Core/SW302</t>
         </is>
       </c>
       <c r="B301" t="inlineStr" s="0">
@@ -18730,7 +18730,7 @@
     <row r="302">
       <c r="A302" t="inlineStr" s="0">
         <is>
-          <t>06_Relay_MasterInhibit/U1</t>
+          <t>06_Relay_MasterInhibit/U601</t>
         </is>
       </c>
       <c r="B302" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Implement ECO-008R TPS2553 current limits
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -11284,7 +11284,7 @@
       </c>
       <c r="S110" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected each TPS2553-Q1 channel to an independent legal 150 kOhm RILIM with calculated 154..209 mA bounds; exact suffix/package, thermal, reverse-current, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
         </is>
       </c>
       <c r="T110" t="inlineStr" s="0">
@@ -11386,7 +11386,7 @@
       </c>
       <c r="S111" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected each TPS2553-Q1 channel to an independent legal 150 kOhm RILIM with calculated 154..209 mA bounds; exact suffix/package, thermal, reverse-current, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
         </is>
       </c>
       <c r="T111" t="inlineStr" s="0">
@@ -11488,7 +11488,7 @@
       </c>
       <c r="S112" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected each TPS2553-Q1 channel to an independent legal 150 kOhm RILIM with calculated 154..209 mA bounds; exact suffix/package, thermal, reverse-current, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
         </is>
       </c>
       <c r="T112" t="inlineStr" s="0">
@@ -25054,7 +25054,7 @@
       </c>
       <c r="S245" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected each TPS2553-Q1 channel to an independent legal 150 kOhm RILIM with calculated 154..209 mA bounds; exact suffix/package, thermal, reverse-current, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
         </is>
       </c>
       <c r="T245" t="inlineStr" s="0">
@@ -25156,7 +25156,7 @@
       </c>
       <c r="S246" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected each TPS2553-Q1 channel to an independent legal 150 kOhm RILIM with calculated 154..209 mA bounds; exact suffix/package, thermal, reverse-current, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
         </is>
       </c>
       <c r="T246" t="inlineStr" s="0">
@@ -25258,7 +25258,7 @@
       </c>
       <c r="S247" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected each TPS2553-Q1 channel to an independent legal 150 kOhm RILIM with calculated 154..209 mA bounds; exact suffix/package, thermal, reverse-current, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
         </is>
       </c>
       <c r="T247" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Complete PAS-01R dependency closure
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -4241,12 +4241,12 @@
       </c>
       <c r="R41" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S41" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Exact DC-bias curve at 55 V after U101/PPC clamp selection.</t>
         </is>
       </c>
       <c r="T41" t="inlineStr" s="0">
@@ -4343,12 +4343,12 @@
       </c>
       <c r="R42" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S42" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Ripple/ESR/lifetime at protected-input waveform.</t>
         </is>
       </c>
       <c r="T42" t="inlineStr" s="0">
@@ -4445,12 +4445,12 @@
       </c>
       <c r="R43" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S43" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Ripple/ESR/lifetime at protected-input waveform.</t>
         </is>
       </c>
       <c r="T43" t="inlineStr" s="0">
@@ -4955,12 +4955,12 @@
       </c>
       <c r="R48" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S48" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Exact DC-bias curve at 55 V after U101/PPC clamp selection.</t>
         </is>
       </c>
       <c r="T48" t="inlineStr" s="0">
@@ -5057,12 +5057,12 @@
       </c>
       <c r="R49" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S49" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” saturation, RMS current, DCR, hot loss, impedance/core loss, and surge evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Impedance/inductance, hot DCR, saturation and loss at protected-input waveform.</t>
         </is>
       </c>
       <c r="T49" t="inlineStr" s="0">
@@ -6791,12 +6791,12 @@
       </c>
       <c r="R66" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S66" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact dielectric, DC-bias effective capacitance, ripple/ESR, aging, and stability evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 WEBENCH input-capacitance and ripple solution.</t>
         </is>
       </c>
       <c r="T66" t="inlineStr" s="0">
@@ -6893,12 +6893,12 @@
       </c>
       <c r="R67" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S67" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: TI requires 100 nF BOOT-to-SW; exact suffix and dielectric check.</t>
         </is>
       </c>
       <c r="T67" t="inlineStr" s="0">
@@ -6995,12 +6995,12 @@
       </c>
       <c r="R68" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S68" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact dielectric, DC-bias effective capacitance, ripple/ESR, aging, and stability evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 integrated-compensation output-capacitance/ESR solution.</t>
         </is>
       </c>
       <c r="T68" t="inlineStr" s="0">
@@ -7097,12 +7097,12 @@
       </c>
       <c r="R69" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S69" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact dielectric, DC-bias effective capacitance, ripple/ESR, aging, and stability evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 integrated-compensation output-capacitance/ESR solution.</t>
         </is>
       </c>
       <c r="T69" t="inlineStr" s="0">
@@ -7199,12 +7199,12 @@
       </c>
       <c r="R70" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S70" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Pin/function reconciliation: selected U201 has internal 4 ms soft start.</t>
         </is>
       </c>
       <c r="T70" t="inlineStr" s="0">
@@ -7301,12 +7301,12 @@
       </c>
       <c r="R71" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S71" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact dielectric, DC-bias effective capacitance, ripple/ESR, aging, and stability evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U202 switchover plus U203 input transient model and exact DC-bias curve.</t>
         </is>
       </c>
       <c r="T71" t="inlineStr" s="0">
@@ -7505,12 +7505,12 @@
       </c>
       <c r="R73" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S73" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact dielectric, DC-bias effective capacitance, ripple/ESR, aging, and stability evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 LC stability and effective-capacitance solution.</t>
         </is>
       </c>
       <c r="T73" t="inlineStr" s="0">
@@ -7607,12 +7607,12 @@
       </c>
       <c r="R74" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S74" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact dielectric, DC-bias effective capacitance, ripple/ESR, aging, and stability evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 LC stability and effective-capacitance solution.</t>
         </is>
       </c>
       <c r="T74" t="inlineStr" s="0">
@@ -7709,12 +7709,12 @@
       </c>
       <c r="R75" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S75" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 exact soft-start equation and tolerance.</t>
         </is>
       </c>
       <c r="T75" t="inlineStr" s="0">
@@ -8933,12 +8933,12 @@
       </c>
       <c r="R87" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S87" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 ripple/current/loss solution at selected PFM/FPWM suffix.</t>
         </is>
       </c>
       <c r="T87" t="inlineStr" s="0">
@@ -9035,12 +9035,12 @@
       </c>
       <c r="R88" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S88" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 exact switching mode, ripple, saturation and loss solution.</t>
         </is>
       </c>
       <c r="T88" t="inlineStr" s="0">
@@ -12707,12 +12707,12 @@
       </c>
       <c r="R124" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S124" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact dielectric, DC-bias effective capacitance, ripple/ESR, aging, and stability evidence are incomplete.</t>
+          <t>PAS-01R: BLOCKED â€” SCHEMATIC ECO REQUIRED. ECO â€” correct CT value/target before selection; required evidence: TPS3890-Q1 full CT tolerance stack and schematic value correction.</t>
         </is>
       </c>
       <c r="T124" t="inlineStr" s="0">
@@ -23927,12 +23927,12 @@
       </c>
       <c r="R234" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
         </is>
       </c>
       <c r="S234" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 physically implemented the fixed 2.7 V, 10 ms supervisor and external 2.930/2.680 V threshold network; exact suffix tolerance, leakage, package, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U801 threshold/hysteresis/leakage full tolerance stack.</t>
         </is>
       </c>
       <c r="T234" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Correct C305 supervisor timing
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -12707,12 +12707,12 @@
       </c>
       <c r="R124" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R; QER-01; PPQ-01; PPQ-02</t>
+          <t>ECO-009; PAS-01R; TPS3890-Q1 SBVS303B</t>
         </is>
       </c>
       <c r="S124" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” SCHEMATIC ECO REQUIRED. ECO â€” correct CT value/target before selection; required evidence: TPS3890-Q1 full CT tolerance stack and schematic value correction.</t>
+          <t>ECO-009 nominal correction complete. BLOCKED pending exact U302 suffix and an accepted minimum/maximum reset-release window; manufacturer/device plus capacitor envelope is approximately 79.1..136.6 ms.</t>
         </is>
       </c>
       <c r="T124" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Close C305 reset-release timing
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -12707,12 +12707,12 @@
       </c>
       <c r="R124" t="inlineStr" s="0">
         <is>
-          <t>ECO-009; PAS-01R; TPS3890-Q1 SBVS303B</t>
+          <t>QER-03 QER-RST-01..08; ECO-009R; PAS-01R; TPS3890-Q1 SBVS303B</t>
         </is>
       </c>
       <c r="S124" t="inlineStr" s="0">
         <is>
-          <t>ECO-009 nominal correction complete. BLOCKED pending exact U302 suffix and an accepted minimum/maximum reset-release window; manufacturer/device plus capacitor envelope is approximately 79.1..136.6 ms.</t>
+          <t>ECO-009R timing implementation verified: 79.1..136.6 ms satisfies QER-03. BLOCKED only for exact U302/C305 MPN, lifecycle, sourcing, and prototype confirmation in PACS-01.</t>
         </is>
       </c>
       <c r="T124" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Audit power active component candidates
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="AVL" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -55,19 +55,19 @@
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="37" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
-    <col min="9" max="9" width="37" customWidth="1"/>
-    <col min="10" max="10" width="31" customWidth="1"/>
+    <col min="9" max="9" width="48" customWidth="1"/>
+    <col min="10" max="10" width="48" customWidth="1"/>
     <col min="11" max="11" width="48" customWidth="1"/>
     <col min="12" max="12" width="48" customWidth="1"/>
     <col min="13" max="13" width="48" customWidth="1"/>
     <col min="14" max="14" width="48" customWidth="1"/>
     <col min="15" max="15" width="34" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="17" max="17" width="32" customWidth="1"/>
     <col min="18" max="18" width="48" customWidth="1"/>
     <col min="19" max="19" width="48" customWidth="1"/>
     <col min="20" max="20" width="13" customWidth="1"/>
@@ -1417,42 +1417,42 @@
       </c>
       <c r="D14" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G14" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="H14" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I14" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K14" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L14" t="inlineStr" s="0">
@@ -1462,12 +1462,12 @@
       </c>
       <c r="M14" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N14" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr" s="0">
@@ -1482,17 +1482,17 @@
       </c>
       <c r="Q14" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R14" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S14" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T14" t="inlineStr" s="0">
@@ -1723,42 +1723,42 @@
       </c>
       <c r="D17" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I17" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K17" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L17" t="inlineStr" s="0">
@@ -1768,12 +1768,12 @@
       </c>
       <c r="M17" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N17" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="O17" t="inlineStr" s="0">
@@ -1788,17 +1788,17 @@
       </c>
       <c r="Q17" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R17" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S17" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T17" t="inlineStr" s="0">
@@ -1825,42 +1825,42 @@
       </c>
       <c r="D18" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I18" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K18" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L18" t="inlineStr" s="0">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="M18" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N18" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr" s="0">
@@ -1890,17 +1890,17 @@
       </c>
       <c r="Q18" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R18" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S18" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T18" t="inlineStr" s="0">
@@ -2029,42 +2029,42 @@
       </c>
       <c r="D20" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TCA9517ADGKR</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G20" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TCA9517ADGKR</t>
         </is>
       </c>
       <c r="H20" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I20" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>PCA9517ADGKR (functional review required)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K20" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L20" t="inlineStr" s="0">
@@ -2074,12 +2074,12 @@
       </c>
       <c r="M20" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N20" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>PCA9517ADGKR (functional review required)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr" s="0">
@@ -2094,17 +2094,17 @@
       </c>
       <c r="Q20" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R20" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S20" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T20" t="inlineStr" s="0">
@@ -2131,42 +2131,42 @@
       </c>
       <c r="D21" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TCA9517ADGKR</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TCA9517ADGKR</t>
         </is>
       </c>
       <c r="H21" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I21" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>PCA9517ADGKR (functional review required)</t>
         </is>
       </c>
       <c r="J21" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K21" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L21" t="inlineStr" s="0">
@@ -2176,12 +2176,12 @@
       </c>
       <c r="M21" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N21" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>PCA9517ADGKR (functional review required)</t>
         </is>
       </c>
       <c r="O21" t="inlineStr" s="0">
@@ -2196,17 +2196,17 @@
       </c>
       <c r="Q21" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R21" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S21" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T21" t="inlineStr" s="0">
@@ -2335,42 +2335,42 @@
       </c>
       <c r="D23" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>SN74LVC1G08QDCKRQ1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>SN74LVC1G08QDCKRQ1</t>
         </is>
       </c>
       <c r="H23" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I23" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>SN74LVC1G08QDRYRQ1 (functional, different package)</t>
         </is>
       </c>
       <c r="J23" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K23" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L23" t="inlineStr" s="0">
@@ -2380,12 +2380,12 @@
       </c>
       <c r="M23" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N23" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>SN74LVC1G08QDRYRQ1 (functional, different package)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr" s="0">
@@ -2400,17 +2400,17 @@
       </c>
       <c r="Q23" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R23" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S23" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC1G08QDCKRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T23" t="inlineStr" s="0">
@@ -2437,42 +2437,42 @@
       </c>
       <c r="D24" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>SN74LVC08AQPWRQ1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>SN74LVC08AQPWRQ1</t>
         </is>
       </c>
       <c r="H24" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I24" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>SN74LVC08AQBQARQ1 (functional, different package)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K24" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L24" t="inlineStr" s="0">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="M24" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N24" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>SN74LVC08AQBQARQ1 (functional, different package)</t>
         </is>
       </c>
       <c r="O24" t="inlineStr" s="0">
@@ -2502,17 +2502,17 @@
       </c>
       <c r="Q24" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R24" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S24" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC08AQPWRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T24" t="inlineStr" s="0">
@@ -2539,42 +2539,42 @@
       </c>
       <c r="D25" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS389030QDSERQ1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS389030QDSERQ1</t>
         </is>
       </c>
       <c r="H25" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I25" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>NONE - threshold/timing/pin exactness required</t>
         </is>
       </c>
       <c r="J25" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K25" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L25" t="inlineStr" s="0">
@@ -2584,12 +2584,12 @@
       </c>
       <c r="M25" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N25" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>NONE - threshold/timing/pin exactness required</t>
         </is>
       </c>
       <c r="O25" t="inlineStr" s="0">
@@ -2604,17 +2604,17 @@
       </c>
       <c r="Q25" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R25" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S25" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS389030QDSERQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T25" t="inlineStr" s="0">
@@ -3559,42 +3559,42 @@
       </c>
       <c r="D35" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>UNRESOLVED - PACS-01 BLOCKED</t>
         </is>
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>NO ACTIVE ORDERABLE TLV841SCPH27YBHR FOUND</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>UNRESOLVED</t>
         </is>
       </c>
       <c r="G35" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>NO ACTIVE ORDERABLE TLV841SCPH27YBHR FOUND</t>
         </is>
       </c>
       <c r="H35" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I35" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Architecture-compatible alternate not demonstrated</t>
         </is>
       </c>
       <c r="J35" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>NOT ORDERABLE / UNRESOLVED</t>
         </is>
       </c>
       <c r="K35" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>UNAVAILABLE / UNRESOLVED</t>
         </is>
       </c>
       <c r="L35" t="inlineStr" s="0">
@@ -3604,12 +3604,12 @@
       </c>
       <c r="M35" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N35" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>Architecture-compatible alternate not demonstrated</t>
         </is>
       </c>
       <c r="O35" t="inlineStr" s="0">
@@ -3624,17 +3624,17 @@
       </c>
       <c r="Q35" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R35" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S35" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 physically implemented the fixed 2.7 V, 10 ms supervisor and external 2.930/2.680 V threshold network; exact suffix tolerance, leakage, package, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-007 physically implemented the fixed 2.7 V, 10 ms supervisor and external 2.930/2.680 V threshold network; exact suffix tolerance, leakage, package, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work. PACS-01 BLOCKED - NO ACTIVE ORDERABLE TLV841SCPH27YBHR FOUND. No active-device freeze.</t>
         </is>
       </c>
       <c r="T35" t="inlineStr" s="0">
@@ -3661,42 +3661,42 @@
       </c>
       <c r="D36" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Infineon</t>
         </is>
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>IAUC100N08S5N034ATMA1</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Infineon</t>
         </is>
       </c>
       <c r="G36" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>IAUC100N08S5N034ATMA1</t>
         </is>
       </c>
       <c r="H36" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I36" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>BUK7J2R4-80M</t>
         </is>
       </c>
       <c r="J36" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K36" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L36" t="inlineStr" s="0">
@@ -3706,12 +3706,12 @@
       </c>
       <c r="M36" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N36" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>BUK7J2R4-80M</t>
         </is>
       </c>
       <c r="O36" t="inlineStr" s="0">
@@ -3726,17 +3726,17 @@
       </c>
       <c r="Q36" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R36" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S36" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts. PACS-01 reviewed candidate IAUC100N08S5N034ATMA1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T36" t="inlineStr" s="0">
@@ -24367,42 +24367,42 @@
       </c>
       <c r="D239" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>UNRESOLVED - PACS-01 BLOCKED</t>
         </is>
       </c>
       <c r="E239" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>UNRESOLVED - CAPTURED TPS26630PWPR IS NOT ORDERABLE</t>
         </is>
       </c>
       <c r="F239" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>UNRESOLVED</t>
         </is>
       </c>
       <c r="G239" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>UNRESOLVED - CAPTURED TPS26630PWPR IS NOT ORDERABLE</t>
         </is>
       </c>
       <c r="H239" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I239" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS26633PWPR requires controlled variant review</t>
         </is>
       </c>
       <c r="J239" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>NOT ORDERABLE / UNRESOLVED</t>
         </is>
       </c>
       <c r="K239" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>UNAVAILABLE / UNRESOLVED</t>
         </is>
       </c>
       <c r="L239" t="inlineStr" s="0">
@@ -24412,12 +24412,12 @@
       </c>
       <c r="M239" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N239" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS26633PWPR requires controlled variant review</t>
         </is>
       </c>
       <c r="O239" t="inlineStr" s="0">
@@ -24432,17 +24432,17 @@
       </c>
       <c r="Q239" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R239" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S239" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 BLOCKED - UNRESOLVED - CAPTURED TPS26630PWPR IS NOT ORDERABLE. No active-device freeze.</t>
         </is>
       </c>
       <c r="T239" t="inlineStr" s="0">
@@ -24469,42 +24469,42 @@
       </c>
       <c r="D240" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E240" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS259470LRPWR</t>
         </is>
       </c>
       <c r="F240" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G240" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS259470LRPWR</t>
         </is>
       </c>
       <c r="H240" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I240" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS259470ARPWR (functional, auto-retry)</t>
         </is>
       </c>
       <c r="J240" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K240" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L240" t="inlineStr" s="0">
@@ -24514,12 +24514,12 @@
       </c>
       <c r="M240" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N240" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS259470ARPWR (functional, auto-retry)</t>
         </is>
       </c>
       <c r="O240" t="inlineStr" s="0">
@@ -24534,17 +24534,17 @@
       </c>
       <c r="Q240" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R240" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S240" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS259470LRPWR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T240" t="inlineStr" s="0">
@@ -24571,42 +24571,42 @@
       </c>
       <c r="D241" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E241" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>LMR38020FSQDDARQ1</t>
         </is>
       </c>
       <c r="F241" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G241" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>LMR38020FSQDDARQ1</t>
         </is>
       </c>
       <c r="H241" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I241" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>LMR38020SQDDARQ1 (functional, PFM)</t>
         </is>
       </c>
       <c r="J241" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K241" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L241" t="inlineStr" s="0">
@@ -24616,12 +24616,12 @@
       </c>
       <c r="M241" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N241" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>LMR38020SQDDARQ1 (functional, PFM)</t>
         </is>
       </c>
       <c r="O241" t="inlineStr" s="0">
@@ -24636,17 +24636,17 @@
       </c>
       <c r="Q241" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R241" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S241" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected the 400 kHz LMR38020F-Q1 RT/SYNC network to 64.9 kOhm; exact suffix, oscillator, loop, loss, thermal, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-007 corrected the 400 kHz LMR38020F-Q1 RT/SYNC network to 64.9 kOhm; exact suffix, oscillator, loop, loss, thermal, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work. PACS-01 reviewed candidate LMR38020FSQDDARQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T241" t="inlineStr" s="0">
@@ -24673,42 +24673,42 @@
       </c>
       <c r="D242" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E242" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2121RUXR</t>
         </is>
       </c>
       <c r="F242" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G242" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2121RUXR</t>
         </is>
       </c>
       <c r="H242" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I242" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2121RUXT (same die, small reel)</t>
         </is>
       </c>
       <c r="J242" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K242" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L242" t="inlineStr" s="0">
@@ -24718,12 +24718,12 @@
       </c>
       <c r="M242" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N242" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS2121RUXT (same die, small reel)</t>
         </is>
       </c>
       <c r="O242" t="inlineStr" s="0">
@@ -24738,17 +24738,17 @@
       </c>
       <c r="Q242" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R242" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S242" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS2121RUXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T242" t="inlineStr" s="0">
@@ -24775,42 +24775,42 @@
       </c>
       <c r="D243" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E243" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS62135RGXR</t>
         </is>
       </c>
       <c r="F243" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G243" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS62135RGXR</t>
         </is>
       </c>
       <c r="H243" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I243" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS621351RGXR (functional, no output discharge)</t>
         </is>
       </c>
       <c r="J243" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K243" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L243" t="inlineStr" s="0">
@@ -24820,12 +24820,12 @@
       </c>
       <c r="M243" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N243" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS621351RGXR (functional, no output discharge)</t>
         </is>
       </c>
       <c r="O243" t="inlineStr" s="0">
@@ -24840,17 +24840,17 @@
       </c>
       <c r="Q243" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R243" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S243" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete.</t>
+          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete. PACS-01 reviewed candidate TPS62135RGXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T243" t="inlineStr" s="0">
@@ -24877,42 +24877,42 @@
       </c>
       <c r="D244" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E244" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="F244" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G244" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="H244" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I244" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="J244" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K244" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L244" t="inlineStr" s="0">
@@ -24922,12 +24922,12 @@
       </c>
       <c r="M244" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N244" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="O244" t="inlineStr" s="0">
@@ -24942,17 +24942,17 @@
       </c>
       <c r="Q244" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R244" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S244" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T244" t="inlineStr" s="0">
@@ -24979,42 +24979,42 @@
       </c>
       <c r="D245" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E245" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2553QDBVRQ1</t>
         </is>
       </c>
       <c r="F245" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G245" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2553QDBVRQ1</t>
         </is>
       </c>
       <c r="H245" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I245" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2551QDBVRQ1 (functional review required)</t>
         </is>
       </c>
       <c r="J245" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K245" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L245" t="inlineStr" s="0">
@@ -25024,12 +25024,12 @@
       </c>
       <c r="M245" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N245" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS2551QDBVRQ1 (functional review required)</t>
         </is>
       </c>
       <c r="O245" t="inlineStr" s="0">
@@ -25044,17 +25044,17 @@
       </c>
       <c r="Q245" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R245" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S245" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T245" t="inlineStr" s="0">
@@ -25081,42 +25081,42 @@
       </c>
       <c r="D246" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E246" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2553QDBVRQ1</t>
         </is>
       </c>
       <c r="F246" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G246" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2553QDBVRQ1</t>
         </is>
       </c>
       <c r="H246" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I246" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2551QDBVRQ1 (functional review required)</t>
         </is>
       </c>
       <c r="J246" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K246" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L246" t="inlineStr" s="0">
@@ -25126,12 +25126,12 @@
       </c>
       <c r="M246" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N246" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS2551QDBVRQ1 (functional review required)</t>
         </is>
       </c>
       <c r="O246" t="inlineStr" s="0">
@@ -25146,17 +25146,17 @@
       </c>
       <c r="Q246" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R246" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S246" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T246" t="inlineStr" s="0">
@@ -25183,42 +25183,42 @@
       </c>
       <c r="D247" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E247" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2553QDBVRQ1</t>
         </is>
       </c>
       <c r="F247" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G247" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2553QDBVRQ1</t>
         </is>
       </c>
       <c r="H247" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I247" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS2551QDBVRQ1 (functional review required)</t>
         </is>
       </c>
       <c r="J247" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K247" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L247" t="inlineStr" s="0">
@@ -25228,12 +25228,12 @@
       </c>
       <c r="M247" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N247" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS2551QDBVRQ1 (functional review required)</t>
         </is>
       </c>
       <c r="O247" t="inlineStr" s="0">
@@ -25248,17 +25248,17 @@
       </c>
       <c r="Q247" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R247" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S247" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T247" t="inlineStr" s="0">
@@ -29977,42 +29977,42 @@
       </c>
       <c r="D294" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E294" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="F294" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G294" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22918TDBVRQ1</t>
         </is>
       </c>
       <c r="H294" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>Functional alternate only</t>
         </is>
       </c>
       <c r="I294" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="J294" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>ACTIVE / PRODUCTION - manufacturer review 2026-07-31</t>
         </is>
       </c>
       <c r="K294" t="inlineStr" s="0">
         <is>
-          <t>NOT REVIEWED - BLOCKED</t>
+          <t>Manufacturer orderable; distributor snapshot requires PO revalidation</t>
         </is>
       </c>
       <c r="L294" t="inlineStr" s="0">
@@ -30022,12 +30022,12 @@
       </c>
       <c r="M294" t="inlineStr" s="0">
         <is>
-          <t>UNRESOLVED - CSR-01A BLOCKED</t>
+          <t>No approved drop-in second source</t>
         </is>
       </c>
       <c r="N294" t="inlineStr" s="0">
         <is>
-          <t/>
+          <t>TPS22995H-Q1 (functional, different pinout)</t>
         </is>
       </c>
       <c r="O294" t="inlineStr" s="0">
@@ -30042,17 +30042,17 @@
       </c>
       <c r="Q294" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED</t>
+          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
         </is>
       </c>
       <c r="R294" t="inlineStr" s="0">
         <is>
-          <t>QER-01; ECO-006; MIR-01 where applicable; CSR-01A-R2 disposition</t>
+          <t>PACS-01; QER-01/02/03; PPQ-01/02; applicable ECO</t>
         </is>
       </c>
       <c r="S294" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
         </is>
       </c>
       <c r="T294" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Revalidate power active component selections
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q17" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R17" t="inlineStr" s="0">
@@ -1798,12 +1798,12 @@
       </c>
       <c r="S17" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts. PACS-01 reviewed candidate IAUC100N08S5N034ATMA1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts. PACS-01 reviewed candidate IAUC100N08S5N034ATMA1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T17" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="Q35" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R SYSTEM REVALIDATION</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R35" t="inlineStr" s="0">
@@ -3634,12 +3634,12 @@
       </c>
       <c r="S35" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS26631PWPR; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release.</t>
+          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS26631PWPR; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T35" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="Q36" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R36" t="inlineStr" s="0">
@@ -3736,12 +3736,12 @@
       </c>
       <c r="S36" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS259470LRPWR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS259470LRPWR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T36" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -10356,7 +10356,7 @@
       </c>
       <c r="Q101" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R101" t="inlineStr" s="0">
@@ -10366,12 +10366,12 @@
       </c>
       <c r="S101" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected the 400 kHz LMR38020F-Q1 RT/SYNC network to 64.9 kOhm; exact suffix, oscillator, loop, loss, thermal, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work. PACS-01 reviewed candidate LMR38020FSQDDARQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-007 corrected the 400 kHz LMR38020F-Q1 RT/SYNC network to 64.9 kOhm; exact suffix, oscillator, loop, loss, thermal, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work. PACS-01 reviewed candidate LMR38020FSQDDARQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T101" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -10458,7 +10458,7 @@
       </c>
       <c r="Q102" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R102" t="inlineStr" s="0">
@@ -10468,12 +10468,12 @@
       </c>
       <c r="S102" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS2121RUXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS2121RUXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T102" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -10560,7 +10560,7 @@
       </c>
       <c r="Q103" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R103" t="inlineStr" s="0">
@@ -10570,12 +10570,12 @@
       </c>
       <c r="S103" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete. PACS-01 reviewed candidate TPS62135RGXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete. PACS-01 reviewed candidate TPS62135RGXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T103" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -10662,7 +10662,7 @@
       </c>
       <c r="Q104" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R104" t="inlineStr" s="0">
@@ -10672,12 +10672,12 @@
       </c>
       <c r="S104" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC1G08QDCKRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC1G08QDCKRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T104" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -10764,7 +10764,7 @@
       </c>
       <c r="Q105" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R105" t="inlineStr" s="0">
@@ -10774,12 +10774,12 @@
       </c>
       <c r="S105" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC08AQPWRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC08AQPWRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T105" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -10866,7 +10866,7 @@
       </c>
       <c r="Q106" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R106" t="inlineStr" s="0">
@@ -10876,12 +10876,12 @@
       </c>
       <c r="S106" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T106" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="Q107" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R107" t="inlineStr" s="0">
@@ -10978,12 +10978,12 @@
       </c>
       <c r="S107" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T107" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -11070,7 +11070,7 @@
       </c>
       <c r="Q108" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R108" t="inlineStr" s="0">
@@ -11080,12 +11080,12 @@
       </c>
       <c r="S108" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T108" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -11172,7 +11172,7 @@
       </c>
       <c r="Q109" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R109" t="inlineStr" s="0">
@@ -11182,12 +11182,12 @@
       </c>
       <c r="S109" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T109" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -11274,7 +11274,7 @@
       </c>
       <c r="Q110" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R110" t="inlineStr" s="0">
@@ -11284,12 +11284,12 @@
       </c>
       <c r="S110" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T110" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -11376,7 +11376,7 @@
       </c>
       <c r="Q111" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R111" t="inlineStr" s="0">
@@ -11386,12 +11386,12 @@
       </c>
       <c r="S111" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T111" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -11478,7 +11478,7 @@
       </c>
       <c r="Q112" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R112" t="inlineStr" s="0">
@@ -11488,12 +11488,12 @@
       </c>
       <c r="S112" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T112" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -11580,7 +11580,7 @@
       </c>
       <c r="Q113" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R113" t="inlineStr" s="0">
@@ -11590,12 +11590,12 @@
       </c>
       <c r="S113" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T113" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -13110,7 +13110,7 @@
       </c>
       <c r="Q128" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R128" t="inlineStr" s="0">
@@ -13120,12 +13120,12 @@
       </c>
       <c r="S128" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS389030QDSERQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS389030QDSERQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T128" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -27390,7 +27390,7 @@
       </c>
       <c r="Q268" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R268" t="inlineStr" s="0">
@@ -27400,12 +27400,12 @@
       </c>
       <c r="S268" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T268" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -27492,7 +27492,7 @@
       </c>
       <c r="Q269" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01 NOT ACCEPTED</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R269" t="inlineStr" s="0">
@@ -27502,12 +27502,12 @@
       </c>
       <c r="S269" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T269" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -30042,7 +30042,7 @@
       </c>
       <c r="Q294" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R SYSTEM REVALIDATION</t>
+          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
         </is>
       </c>
       <c r="R294" t="inlineStr" s="0">
@@ -30052,12 +30052,12 @@
       </c>
       <c r="S294" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS3899DL01DSER; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release.</t>
+          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS3899DL01DSER; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
         </is>
       </c>
       <c r="T294" t="inlineStr" s="0">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close stale PACS passive dependencies
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -370,7 +370,7 @@
       </c>
       <c r="S3" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Exact DC-bias curve at 55 V after U101/PPC clamp selection.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T3" t="inlineStr" s="0">
@@ -472,7 +472,7 @@
       </c>
       <c r="S4" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Ripple/ESR/lifetime at protected-input waveform.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T4" t="inlineStr" s="0">
@@ -574,7 +574,7 @@
       </c>
       <c r="S5" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Ripple/ESR/lifetime at protected-input waveform.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T5" t="inlineStr" s="0">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="S10" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Exact DC-bias curve at 55 V after U101/PPC clamp selection.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T10" t="inlineStr" s="0">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="S16" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Impedance/inductance, hot DCR, saturation and loss at protected-input waveform.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T16" t="inlineStr" s="0">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="S37" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 WEBENCH input-capacitance and ripple solution.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T37" t="inlineStr" s="0">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="S38" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: TI requires 100 nF BOOT-to-SW; exact suffix and dielectric check.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T38" t="inlineStr" s="0">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="S39" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 integrated-compensation output-capacitance/ESR solution.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T39" t="inlineStr" s="0">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="S40" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 integrated-compensation output-capacitance/ESR solution.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T40" t="inlineStr" s="0">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="S41" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: Pin/function reconciliation: selected U201 has internal 4 ms soft start.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T41" t="inlineStr" s="0">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="S42" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U202 switchover plus U203 input transient model and exact DC-bias curve.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T42" t="inlineStr" s="0">
@@ -4552,7 +4552,7 @@
       </c>
       <c r="S44" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 LC stability and effective-capacitance solution.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T44" t="inlineStr" s="0">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="S45" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 LC stability and effective-capacitance solution.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T45" t="inlineStr" s="0">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="S46" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 exact soft-start equation and tolerance.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T46" t="inlineStr" s="0">
@@ -7000,7 +7000,7 @@
       </c>
       <c r="S68" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U201 ripple/current/loss solution at selected PFM/FPWM suffix.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T68" t="inlineStr" s="0">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="S69" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. PACS-01 â€” freeze named active, then execute official tool/curve check; required evidence: U203 exact switching mode, ripple, saturation and loss solution.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T69" t="inlineStr" s="0">
@@ -28012,7 +28012,7 @@
       </c>
       <c r="S274" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. ECO-010 support element requires exact passive selection after PACS-01R.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T274" t="inlineStr" s="0">
@@ -29134,7 +29134,7 @@
       </c>
       <c r="S285" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. ECO-010 support element requires exact passive selection after PACS-01R.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T285" t="inlineStr" s="0">
@@ -29236,7 +29236,7 @@
       </c>
       <c r="S286" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. ECO-010 support element requires exact passive selection after PACS-01R.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T286" t="inlineStr" s="0">
@@ -29338,7 +29338,7 @@
       </c>
       <c r="S287" t="inlineStr" s="0">
         <is>
-          <t>PAS-01R: BLOCKED â€” ACTIVE DEVICE SELECTION REQUIRED. ECO-010 support element requires exact passive selection after PACS-01R.</t>
+          <t>PAS-01R: BLOCKED - exact active MPN selected; named manufacturer tool/curve, thermal, magnetic or threshold evidence remains under PACS-01R-A.</t>
         </is>
       </c>
       <c r="T287" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Control external active evidence acquisition
</commit_message>
<xml_diff>
--- a/docs/bom/Approved_Vendor_List.xlsx
+++ b/docs/bom/Approved_Vendor_List.xlsx
@@ -67,7 +67,7 @@
     <col min="14" max="14" width="48" customWidth="1"/>
     <col min="15" max="15" width="34" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
-    <col min="17" max="17" width="40" customWidth="1"/>
+    <col min="17" max="17" width="41" customWidth="1"/>
     <col min="18" max="18" width="48" customWidth="1"/>
     <col min="19" max="19" width="48" customWidth="1"/>
     <col min="20" max="20" width="13" customWidth="1"/>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="Q17" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R17" t="inlineStr" s="0">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="S17" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts. PACS-01 reviewed candidate IAUC100N08S5N034ATMA1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 corrected the electrical class; exact manufacturer curve, tolerance, thermal/SOA, lifecycle, sourcing, and cost evidence remain pending after CSR-01A-R2 stopped on released-network conflicts. PACS-01 reviewed candidate IAUC100N08S5N034ATMA1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T17" t="inlineStr" s="0">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="Q35" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R35" t="inlineStr" s="0">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="S35" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS26631PWPR; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS26631PWPR; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T35" t="inlineStr" s="0">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="Q36" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R36" t="inlineStr" s="0">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="S36" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS259470LRPWR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS259470LRPWR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T36" t="inlineStr" s="0">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="Q101" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R101" t="inlineStr" s="0">
@@ -10366,7 +10366,7 @@
       </c>
       <c r="S101" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-007 corrected the 400 kHz LMR38020F-Q1 RT/SYNC network to 64.9 kOhm; exact suffix, oscillator, loop, loss, thermal, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work. PACS-01 reviewed candidate LMR38020FSQDDARQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-007 corrected the 400 kHz LMR38020F-Q1 RT/SYNC network to 64.9 kOhm; exact suffix, oscillator, loop, loss, thermal, lifecycle, sourcing, and cost evidence remain CSR-01A-R3 work. PACS-01 reviewed candidate LMR38020FSQDDARQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T101" t="inlineStr" s="0">
@@ -10458,7 +10458,7 @@
       </c>
       <c r="Q102" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R102" t="inlineStr" s="0">
@@ -10468,7 +10468,7 @@
       </c>
       <c r="S102" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS2121RUXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS2121RUXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T102" t="inlineStr" s="0">
@@ -10560,7 +10560,7 @@
       </c>
       <c r="Q103" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R103" t="inlineStr" s="0">
@@ -10570,7 +10570,7 @@
       </c>
       <c r="S103" t="inlineStr" s="0">
         <is>
-          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete. PACS-01 reviewed candidate TPS62135RGXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>THERMAL/STABILITY EVIDENCE MISSING â€” vendor-tool, effective-capacitance, loop/stability, loss, and minimum-copper analysis are incomplete. PACS-01 reviewed candidate TPS62135RGXR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T103" t="inlineStr" s="0">
@@ -10662,7 +10662,7 @@
       </c>
       <c r="Q104" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R104" t="inlineStr" s="0">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="S104" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC1G08QDCKRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC1G08QDCKRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T104" t="inlineStr" s="0">
@@ -10764,7 +10764,7 @@
       </c>
       <c r="Q105" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R105" t="inlineStr" s="0">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="S105" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC08AQPWRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate SN74LVC08AQPWRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T105" t="inlineStr" s="0">
@@ -10866,7 +10866,7 @@
       </c>
       <c r="Q106" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R106" t="inlineStr" s="0">
@@ -10876,7 +10876,7 @@
       </c>
       <c r="S106" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T106" t="inlineStr" s="0">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="Q107" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R107" t="inlineStr" s="0">
@@ -10978,7 +10978,7 @@
       </c>
       <c r="S107" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T107" t="inlineStr" s="0">
@@ -11070,7 +11070,7 @@
       </c>
       <c r="Q108" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R108" t="inlineStr" s="0">
@@ -11080,7 +11080,7 @@
       </c>
       <c r="S108" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T108" t="inlineStr" s="0">
@@ -11172,7 +11172,7 @@
       </c>
       <c r="Q109" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R109" t="inlineStr" s="0">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="S109" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T109" t="inlineStr" s="0">
@@ -11274,7 +11274,7 @@
       </c>
       <c r="Q110" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R110" t="inlineStr" s="0">
@@ -11284,7 +11284,7 @@
       </c>
       <c r="S110" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T110" t="inlineStr" s="0">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="Q111" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R111" t="inlineStr" s="0">
@@ -11386,7 +11386,7 @@
       </c>
       <c r="S111" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS22918TDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T111" t="inlineStr" s="0">
@@ -11478,7 +11478,7 @@
       </c>
       <c r="Q112" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R112" t="inlineStr" s="0">
@@ -11488,7 +11488,7 @@
       </c>
       <c r="S112" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T112" t="inlineStr" s="0">
@@ -11580,7 +11580,7 @@
       </c>
       <c r="Q113" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R113" t="inlineStr" s="0">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="S113" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE - ECO-008R implements a generic 141 kOhm +/-1%, &lt;=100 ppm/degC RILIM with calculated 162.8..222.4 mA bounds under QER-02; exact MPN/suffix/package, thermal, reverse-current, lifecycle, sourcing, cost, and prototype evidence remain CSR-01A-R4 work. PACS-01 reviewed candidate TPS2553QDBVRQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T113" t="inlineStr" s="0">
@@ -13110,7 +13110,7 @@
       </c>
       <c r="Q128" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R128" t="inlineStr" s="0">
@@ -13120,7 +13120,7 @@
       </c>
       <c r="S128" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS389030QDSERQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” exact suffix equations, pin mapping, thresholds, timing, partial-power, thermal, and fault behavior are not all closed. PACS-01 reviewed candidate TPS389030QDSERQ1; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T128" t="inlineStr" s="0">
@@ -27390,7 +27390,7 @@
       </c>
       <c r="Q268" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R268" t="inlineStr" s="0">
@@ -27400,7 +27400,7 @@
       </c>
       <c r="S268" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T268" t="inlineStr" s="0">
@@ -27492,7 +27492,7 @@
       </c>
       <c r="Q269" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R269" t="inlineStr" s="0">
@@ -27502,7 +27502,7 @@
       </c>
       <c r="S269" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE â€” ECO-006 physical class is defined and TCA9517A is a candidate; exact pin equivalence, offset-low compatibility, partial-power behavior, lifecycle, sourcing, and cost evidence remain pending. PACS-01 reviewed candidate TCA9517ADGKR; package rejected as a whole because U101 and U801 remain blocked. Do not procure or assign footprint. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T269" t="inlineStr" s="0">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="Q294" t="inlineStr" s="0">
         <is>
-          <t>BLOCKED - PACS-01R-A EVIDENCE CLOSURE</t>
+          <t>BLOCKED - EXTERNAL EVIDENCE ACQUISITION</t>
         </is>
       </c>
       <c r="R294" t="inlineStr" s="0">
@@ -30052,7 +30052,7 @@
       </c>
       <c r="S294" t="inlineStr" s="0">
         <is>
-          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS3899DL01DSER; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required.</t>
+          <t>ANALYSIS INCOMPLETE - exact suffix/system revalidation remains required. ECO-010 selectable implementation TPS3899DL01DSER; BLOCKED - PACS-01R SYSTEM REVALIDATION; no footprint or procurement release. PACS-01R: BLOCKED - exact active candidate retained; thermal/tool, dependent-passive, prototype, alternate, and current commercial evidence closure required. PACS-01R-B1R-X: external tool, authoritative thermal and authenticated commercial artifacts remain open; see docs/evidence/External_Evidence_Acquisition_Inventory.csv.</t>
         </is>
       </c>
       <c r="T294" t="inlineStr" s="0">

</xml_diff>